<commit_message>
Balance termico: se sacan los parentesis vacios de las paredes
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01NNMcFTBbEuLfDho1wCZzu7
</commit_message>
<xml_diff>
--- a/planillas/planillas_estructura (para AutoCAD).xlsx
+++ b/planillas/planillas_estructura (para AutoCAD).xlsx
@@ -20481,7 +20481,7 @@
       <c r="A41" s="47" t="n"/>
       <c r="B41" s="81" t="inlineStr">
         <is>
-          <t>AISLADAS (    )</t>
+          <t>AISLADAS</t>
         </is>
       </c>
       <c r="C41" s="18" t="n"/>
@@ -20496,7 +20496,7 @@
       <c r="A42" s="47" t="n"/>
       <c r="B42" s="81" t="inlineStr">
         <is>
-          <t>INTERIORES (    )</t>
+          <t>INTERIORES</t>
         </is>
       </c>
       <c r="C42" s="18" t="inlineStr">
@@ -20542,7 +20542,7 @@
       <c r="A44" s="50" t="n"/>
       <c r="B44" s="82" t="inlineStr">
         <is>
-          <t>INTERIORES (    )</t>
+          <t>INTERIORES</t>
         </is>
       </c>
       <c r="C44" s="18" t="inlineStr">
@@ -21045,7 +21045,7 @@
       <c r="A71" s="47" t="n"/>
       <c r="B71" s="81" t="inlineStr">
         <is>
-          <t>AISLADAS ()</t>
+          <t>AISLADAS</t>
         </is>
       </c>
       <c r="C71" s="18" t="inlineStr">
@@ -21068,7 +21068,7 @@
       <c r="A72" s="47" t="n"/>
       <c r="B72" s="81" t="inlineStr">
         <is>
-          <t>INTERIORES (    )</t>
+          <t>INTERIORES</t>
         </is>
       </c>
       <c r="C72" s="18" t="inlineStr">
@@ -21091,7 +21091,7 @@
       <c r="A73" s="50" t="n"/>
       <c r="B73" s="82" t="inlineStr">
         <is>
-          <t>INTERIORES (    )</t>
+          <t>INTERIORES</t>
         </is>
       </c>
       <c r="C73" s="18" t="inlineStr">
@@ -21495,7 +21495,7 @@
       <c r="A95" s="43" t="n"/>
       <c r="B95" s="79" t="inlineStr">
         <is>
-          <t>AISLADAS ()</t>
+          <t>AISLADAS</t>
         </is>
       </c>
       <c r="C95" s="18" t="inlineStr">
@@ -21518,7 +21518,7 @@
       <c r="A96" s="47" t="n"/>
       <c r="B96" s="81" t="inlineStr">
         <is>
-          <t>AISLADAS (    )</t>
+          <t>AISLADAS</t>
         </is>
       </c>
       <c r="C96" s="18" t="n"/>
@@ -21556,7 +21556,7 @@
       <c r="A98" s="47" t="n"/>
       <c r="B98" s="81" t="inlineStr">
         <is>
-          <t>INTERIORES (    )</t>
+          <t>INTERIORES</t>
         </is>
       </c>
       <c r="C98" s="18" t="inlineStr">
@@ -21579,7 +21579,7 @@
       <c r="A99" s="47" t="n"/>
       <c r="B99" s="81" t="inlineStr">
         <is>
-          <t>INTERIORES (    )</t>
+          <t>INTERIORES</t>
         </is>
       </c>
       <c r="C99" s="18" t="inlineStr">
@@ -21602,7 +21602,7 @@
       <c r="A100" s="47" t="n"/>
       <c r="B100" s="81" t="inlineStr">
         <is>
-          <t>INTERIORES (    )</t>
+          <t>INTERIORES</t>
         </is>
       </c>
       <c r="C100" s="18" t="inlineStr">
@@ -21625,7 +21625,7 @@
       <c r="A101" s="47" t="n"/>
       <c r="B101" s="81" t="inlineStr">
         <is>
-          <t>INTERIORES (    )</t>
+          <t>INTERIORES</t>
         </is>
       </c>
       <c r="C101" s="18" t="inlineStr">
@@ -21648,7 +21648,7 @@
       <c r="A102" s="50" t="n"/>
       <c r="B102" s="82" t="inlineStr">
         <is>
-          <t>INTERIORES (    )</t>
+          <t>INTERIORES</t>
         </is>
       </c>
       <c r="C102" s="18" t="inlineStr">
@@ -22122,7 +22122,7 @@
       <c r="A128" s="43" t="n"/>
       <c r="B128" s="79" t="inlineStr">
         <is>
-          <t>AISLADAS ()</t>
+          <t>AISLADAS</t>
         </is>
       </c>
       <c r="C128" s="18" t="inlineStr">
@@ -22145,7 +22145,7 @@
       <c r="A129" s="47" t="n"/>
       <c r="B129" s="81" t="inlineStr">
         <is>
-          <t>AISLADAS ()</t>
+          <t>AISLADAS</t>
         </is>
       </c>
       <c r="C129" s="18" t="inlineStr">
@@ -22168,7 +22168,7 @@
       <c r="A130" s="47" t="n"/>
       <c r="B130" s="81" t="inlineStr">
         <is>
-          <t>INTERIORES (    )</t>
+          <t>INTERIORES</t>
         </is>
       </c>
       <c r="C130" s="18" t="inlineStr">
@@ -22191,7 +22191,7 @@
       <c r="A131" s="50" t="n"/>
       <c r="B131" s="82" t="inlineStr">
         <is>
-          <t>INTERIORES (    )</t>
+          <t>INTERIORES</t>
         </is>
       </c>
       <c r="C131" s="18" t="inlineStr">
@@ -22672,7 +22672,7 @@
       <c r="A156" s="47" t="n"/>
       <c r="B156" s="81" t="inlineStr">
         <is>
-          <t>AISLADAS ()</t>
+          <t>AISLADAS</t>
         </is>
       </c>
       <c r="C156" s="18" t="inlineStr">
@@ -22695,7 +22695,7 @@
       <c r="A157" s="47" t="n"/>
       <c r="B157" s="81" t="inlineStr">
         <is>
-          <t>INTERIORES (    )</t>
+          <t>INTERIORES</t>
         </is>
       </c>
       <c r="C157" s="18" t="inlineStr">
@@ -22718,7 +22718,7 @@
       <c r="A158" s="50" t="n"/>
       <c r="B158" s="82" t="inlineStr">
         <is>
-          <t>INTERIORES (    )</t>
+          <t>INTERIORES</t>
         </is>
       </c>
       <c r="C158" s="18" t="n"/>
@@ -23207,7 +23207,7 @@
       <c r="A185" s="47" t="n"/>
       <c r="B185" s="81" t="inlineStr">
         <is>
-          <t>AISLADAS (    )</t>
+          <t>AISLADAS</t>
         </is>
       </c>
       <c r="C185" s="18" t="n"/>
@@ -23222,7 +23222,7 @@
       <c r="A186" s="47" t="n"/>
       <c r="B186" s="81" t="inlineStr">
         <is>
-          <t>INTERIORES (    )</t>
+          <t>INTERIORES</t>
         </is>
       </c>
       <c r="C186" s="18" t="inlineStr">
@@ -23245,7 +23245,7 @@
       <c r="A187" s="47" t="n"/>
       <c r="B187" s="81" t="inlineStr">
         <is>
-          <t>INTERIORES (    )</t>
+          <t>INTERIORES</t>
         </is>
       </c>
       <c r="C187" s="18" t="inlineStr">
@@ -23268,7 +23268,7 @@
       <c r="A188" s="50" t="n"/>
       <c r="B188" s="82" t="inlineStr">
         <is>
-          <t>INTERIORES (    )</t>
+          <t>INTERIORES</t>
         </is>
       </c>
       <c r="C188" s="18" t="inlineStr">
@@ -23734,7 +23734,7 @@
       <c r="A214" s="43" t="n"/>
       <c r="B214" s="79" t="inlineStr">
         <is>
-          <t>AISLADAS ()</t>
+          <t>AISLADAS</t>
         </is>
       </c>
       <c r="C214" s="18" t="inlineStr">
@@ -23757,7 +23757,7 @@
       <c r="A215" s="47" t="n"/>
       <c r="B215" s="81" t="inlineStr">
         <is>
-          <t>AISLADAS (    )</t>
+          <t>AISLADAS</t>
         </is>
       </c>
       <c r="C215" s="18" t="n"/>
@@ -23772,7 +23772,7 @@
       <c r="A216" s="47" t="n"/>
       <c r="B216" s="81" t="inlineStr">
         <is>
-          <t>INTERIORES (    )</t>
+          <t>INTERIORES</t>
         </is>
       </c>
       <c r="C216" s="18" t="inlineStr">
@@ -23795,7 +23795,7 @@
       <c r="A217" s="47" t="n"/>
       <c r="B217" s="81" t="inlineStr">
         <is>
-          <t>INTERIORES (    )</t>
+          <t>INTERIORES</t>
         </is>
       </c>
       <c r="C217" s="18" t="inlineStr">
@@ -23818,7 +23818,7 @@
       <c r="A218" s="50" t="n"/>
       <c r="B218" s="82" t="inlineStr">
         <is>
-          <t>INTERIORES (    )</t>
+          <t>INTERIORES</t>
         </is>
       </c>
       <c r="C218" s="18" t="inlineStr">
@@ -24361,7 +24361,7 @@
       <c r="A247" s="47" t="n"/>
       <c r="B247" s="81" t="inlineStr">
         <is>
-          <t>AISLADAS ()</t>
+          <t>AISLADAS</t>
         </is>
       </c>
       <c r="C247" s="18" t="inlineStr">
@@ -24384,7 +24384,7 @@
       <c r="A248" s="47" t="n"/>
       <c r="B248" s="81" t="inlineStr">
         <is>
-          <t>INTERIORES (    )</t>
+          <t>INTERIORES</t>
         </is>
       </c>
       <c r="C248" s="18" t="inlineStr">
@@ -24407,7 +24407,7 @@
       <c r="A249" s="50" t="n"/>
       <c r="B249" s="82" t="inlineStr">
         <is>
-          <t>INTERIORES (    )</t>
+          <t>INTERIORES</t>
         </is>
       </c>
       <c r="C249" s="18" t="n"/>
@@ -24896,7 +24896,7 @@
       <c r="A276" s="47" t="n"/>
       <c r="B276" s="81" t="inlineStr">
         <is>
-          <t>AISLADAS (    )</t>
+          <t>AISLADAS</t>
         </is>
       </c>
       <c r="C276" s="18" t="n"/>
@@ -24911,7 +24911,7 @@
       <c r="A277" s="47" t="n"/>
       <c r="B277" s="81" t="inlineStr">
         <is>
-          <t>INTERIORES (    )</t>
+          <t>INTERIORES</t>
         </is>
       </c>
       <c r="C277" s="18" t="inlineStr">
@@ -24934,7 +24934,7 @@
       <c r="A278" s="47" t="n"/>
       <c r="B278" s="81" t="inlineStr">
         <is>
-          <t>INTERIORES (    )</t>
+          <t>INTERIORES</t>
         </is>
       </c>
       <c r="C278" s="18" t="inlineStr">
@@ -24957,7 +24957,7 @@
       <c r="A279" s="50" t="n"/>
       <c r="B279" s="82" t="inlineStr">
         <is>
-          <t>INTERIORES (    )</t>
+          <t>INTERIORES</t>
         </is>
       </c>
       <c r="C279" s="18" t="inlineStr">
@@ -25460,7 +25460,7 @@
       <c r="A306" s="47" t="n"/>
       <c r="B306" s="81" t="inlineStr">
         <is>
-          <t>AISLADAS ()</t>
+          <t>AISLADAS</t>
         </is>
       </c>
       <c r="C306" s="18" t="inlineStr">
@@ -25483,7 +25483,7 @@
       <c r="A307" s="47" t="n"/>
       <c r="B307" s="81" t="inlineStr">
         <is>
-          <t>INTERIORES (    )</t>
+          <t>INTERIORES</t>
         </is>
       </c>
       <c r="C307" s="18" t="inlineStr">
@@ -25506,7 +25506,7 @@
       <c r="A308" s="50" t="n"/>
       <c r="B308" s="82" t="inlineStr">
         <is>
-          <t>INTERIORES (    )</t>
+          <t>INTERIORES</t>
         </is>
       </c>
       <c r="C308" s="18" t="inlineStr">
@@ -25980,7 +25980,7 @@
       <c r="A334" s="43" t="n"/>
       <c r="B334" s="79" t="inlineStr">
         <is>
-          <t>AISLADAS ()</t>
+          <t>AISLADAS</t>
         </is>
       </c>
       <c r="C334" s="18" t="inlineStr">
@@ -26003,7 +26003,7 @@
       <c r="A335" s="47" t="n"/>
       <c r="B335" s="81" t="inlineStr">
         <is>
-          <t>AISLADAS ()</t>
+          <t>AISLADAS</t>
         </is>
       </c>
       <c r="C335" s="18" t="inlineStr">
@@ -26026,7 +26026,7 @@
       <c r="A336" s="47" t="n"/>
       <c r="B336" s="81" t="inlineStr">
         <is>
-          <t>INTERIORES (    )</t>
+          <t>INTERIORES</t>
         </is>
       </c>
       <c r="C336" s="18" t="inlineStr">
@@ -26049,7 +26049,7 @@
       <c r="A337" s="50" t="n"/>
       <c r="B337" s="82" t="inlineStr">
         <is>
-          <t>INTERIORES (    )</t>
+          <t>INTERIORES</t>
         </is>
       </c>
       <c r="C337" s="18" t="inlineStr">

</xml_diff>

<commit_message>
Balance termico: living comedor, paredes interiores con cocina y escalera
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01NNMcFTBbEuLfDho1wCZzu7
</commit_message>
<xml_diff>
--- a/planillas/planillas_estructura (para AutoCAD).xlsx
+++ b/planillas/planillas_estructura (para AutoCAD).xlsx
@@ -20496,7 +20496,7 @@
       <c r="A42" s="47" t="n"/>
       <c r="B42" s="81" t="inlineStr">
         <is>
-          <t>INTERIORES</t>
+          <t>INTERIORES (cocina)</t>
         </is>
       </c>
       <c r="C42" s="18" t="inlineStr">
@@ -20542,7 +20542,7 @@
       <c r="A44" s="50" t="n"/>
       <c r="B44" s="82" t="inlineStr">
         <is>
-          <t>INTERIORES</t>
+          <t>INTERIORES (escalera)</t>
         </is>
       </c>
       <c r="C44" s="18" t="inlineStr">

</xml_diff>

<commit_message>
Hall de ingreso: 4,00 x 2,15 y paredes con vestidor, patio interior y living
Se corrigen las medidas en el balance termico y en la planilla de
iluminacion y ventilacion (8,60 m2).

Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01NNMcFTBbEuLfDho1wCZzu7
</commit_message>
<xml_diff>
--- a/planillas/planillas_estructura (para AutoCAD).xlsx
+++ b/planillas/planillas_estructura (para AutoCAD).xlsx
@@ -1645,26 +1645,26 @@
       </c>
       <c r="L8" s="20" t="n"/>
     </row>
-    <row r="9" ht="47" customHeight="1">
+    <row r="9" ht="62" customHeight="1">
       <c r="A9" s="25" t="inlineStr">
         <is>
           <t>07 - Hall / ingreso</t>
         </is>
       </c>
       <c r="B9" s="16" t="n">
-        <v>3.52</v>
+        <v>4</v>
       </c>
       <c r="C9" s="26" t="n">
         <v>2.15</v>
       </c>
       <c r="D9" s="19" t="n">
-        <v>7.568</v>
+        <v>8.6</v>
       </c>
       <c r="E9" s="18" t="n">
         <v>9</v>
       </c>
       <c r="F9" s="19" t="n">
-        <v>0.840888888888889</v>
+        <v>0.955555555555556</v>
       </c>
       <c r="G9" s="19" t="n">
         <v>10.5</v>
@@ -1675,7 +1675,7 @@
         </is>
       </c>
       <c r="I9" s="19" t="n">
-        <v>0.280296296296296</v>
+        <v>0.318518518518519</v>
       </c>
       <c r="J9" s="19" t="n">
         <v>1.6</v>
@@ -1687,7 +1687,7 @@
       </c>
       <c r="L9" s="23" t="inlineStr">
         <is>
-          <t>CORREGIDO: la planilla original repetia los valores del local 03 (0,66 y 0,22). Con 7,53 m2 corresponden 0,84 y 0,28. Cumple igual.</t>
+          <t>CORREGIDO: la planilla original repetia los valores del local 03 (0,66 y 0,22). Con 4,00 x 2,15 = 8,60 m2 corresponden 0,96 y 0,32. Cumple igual.</t>
         </is>
       </c>
     </row>
@@ -5263,7 +5263,7 @@
       <c r="A8" s="116" t="n"/>
       <c r="B8" s="117" t="inlineStr">
         <is>
-          <t>valores del local 03 (Lavadero, 6,0 m2). Con sus 3,50 x 2,15 = 7,53 m2 corresponden</t>
+          <t>valores del local 03 (Lavadero, 6,0 m2). Con sus 4,00 x 2,15 = 8,60 m2 corresponden</t>
         </is>
       </c>
     </row>
@@ -5271,7 +5271,7 @@
       <c r="A9" s="116" t="n"/>
       <c r="B9" s="117" t="inlineStr">
         <is>
-          <t>0,84 y 0,28. No cambia el resultado, pero el numero no cerraba con la superficie</t>
+          <t>0,96 y 0,32. No cambia el resultado, pero el numero no cerraba con la superficie</t>
         </is>
       </c>
     </row>
@@ -20817,7 +20817,7 @@
       <c r="D58" s="12" t="n"/>
       <c r="E58" s="39" t="n"/>
       <c r="F58" s="87" t="n">
-        <v>1924.1</v>
+        <v>2050.7</v>
       </c>
       <c r="G58" s="53" t="n"/>
     </row>
@@ -20832,7 +20832,7 @@
       <c r="D59" s="12" t="n"/>
       <c r="E59" s="14" t="n"/>
       <c r="F59" s="85" t="n">
-        <v>7649.7</v>
+        <v>7776.3</v>
       </c>
       <c r="G59" s="53" t="n"/>
     </row>
@@ -20876,7 +20876,7 @@
         </is>
       </c>
       <c r="C62" s="59" t="n">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="D62" s="12" t="n"/>
       <c r="E62" s="39" t="n"/>
@@ -20891,7 +20891,7 @@
         </is>
       </c>
       <c r="C63" s="59" t="n">
-        <v>224</v>
+        <v>232</v>
       </c>
       <c r="D63" s="12" t="n"/>
       <c r="E63" s="39" t="n"/>
@@ -21027,17 +21027,17 @@
       </c>
       <c r="C70" s="18" t="inlineStr">
         <is>
-          <t>3.52 x 3.00</t>
+          <t>4.00 x 3.00</t>
         </is>
       </c>
       <c r="D70" s="19" t="n">
-        <v>10.56</v>
+        <v>12</v>
       </c>
       <c r="E70" s="59" t="n">
         <v>20</v>
       </c>
       <c r="F70" s="80" t="n">
-        <v>211.2</v>
+        <v>240</v>
       </c>
       <c r="G70" s="53" t="n"/>
     </row>
@@ -21068,22 +21068,22 @@
       <c r="A72" s="47" t="n"/>
       <c r="B72" s="81" t="inlineStr">
         <is>
-          <t>INTERIORES</t>
+          <t>INTERIORES (vestidor)</t>
         </is>
       </c>
       <c r="C72" s="18" t="inlineStr">
         <is>
-          <t>3.52 x 3.00</t>
+          <t>4.00 x 3.00</t>
         </is>
       </c>
       <c r="D72" s="19" t="n">
-        <v>10.56</v>
+        <v>12</v>
       </c>
       <c r="E72" s="59" t="n">
         <v>25</v>
       </c>
       <c r="F72" s="80" t="n">
-        <v>264</v>
+        <v>300</v>
       </c>
       <c r="G72" s="53" t="n"/>
     </row>
@@ -21091,7 +21091,7 @@
       <c r="A73" s="50" t="n"/>
       <c r="B73" s="82" t="inlineStr">
         <is>
-          <t>INTERIORES</t>
+          <t>INTERIORES (living comedor)</t>
         </is>
       </c>
       <c r="C73" s="18" t="inlineStr">
@@ -21170,13 +21170,13 @@
         </is>
       </c>
       <c r="D77" s="19" t="n">
-        <v>7.57</v>
+        <v>8.6</v>
       </c>
       <c r="E77" s="59" t="n">
         <v>15</v>
       </c>
       <c r="F77" s="80" t="n">
-        <v>113.6</v>
+        <v>129</v>
       </c>
       <c r="G77" s="53" t="n"/>
     </row>
@@ -21210,13 +21210,13 @@
         </is>
       </c>
       <c r="D79" s="19" t="n">
-        <v>7.57</v>
+        <v>8.6</v>
       </c>
       <c r="E79" s="59" t="n">
         <v>10</v>
       </c>
       <c r="F79" s="80" t="n">
-        <v>75.7</v>
+        <v>86</v>
       </c>
       <c r="G79" s="53" t="n"/>
     </row>
@@ -21280,17 +21280,17 @@
       </c>
       <c r="C83" s="18" t="inlineStr">
         <is>
-          <t>7.57 m2 x 3.00</t>
+          <t>8.60 m2 x 3.00</t>
         </is>
       </c>
       <c r="D83" s="19" t="n">
-        <v>22.71</v>
+        <v>25.8</v>
       </c>
       <c r="E83" s="59" t="n">
         <v>9</v>
       </c>
       <c r="F83" s="80" t="n">
-        <v>204.4</v>
+        <v>232.2</v>
       </c>
       <c r="G83" s="53" t="n"/>
     </row>
@@ -21324,7 +21324,7 @@
       <c r="D85" s="18" t="n"/>
       <c r="E85" s="20" t="n"/>
       <c r="F85" s="85" t="n">
-        <v>1798.2</v>
+        <v>1916.5</v>
       </c>
       <c r="G85" s="53" t="n"/>
     </row>
@@ -21341,13 +21341,13 @@
       </c>
       <c r="C86" s="47" t="inlineStr">
         <is>
-          <t>1798.20  X  1.07 (FI)  X  1 (FO)  X  1 (FZ)</t>
+          <t>1916.50  X  1.07 (FI)  X  1 (FO)  X  1 (FZ)</t>
         </is>
       </c>
       <c r="D86" s="12" t="n"/>
       <c r="E86" s="14" t="n"/>
       <c r="F86" s="85" t="n">
-        <v>1924.1</v>
+        <v>2050.7</v>
       </c>
       <c r="G86" s="53" t="n"/>
     </row>
@@ -21375,7 +21375,7 @@
       <c r="D88" s="12" t="n"/>
       <c r="E88" s="14" t="n"/>
       <c r="F88" s="85" t="n">
-        <v>1924.1</v>
+        <v>2050.7</v>
       </c>
       <c r="G88" s="53" t="n"/>
     </row>

</xml_diff>

<commit_message>
Balance termico: orientacion en las paredes interiores donde sale de la pared opuesta
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01NNMcFTBbEuLfDho1wCZzu7
</commit_message>
<xml_diff>
--- a/planillas/planillas_estructura (para AutoCAD).xlsx
+++ b/planillas/planillas_estructura (para AutoCAD).xlsx
@@ -19938,7 +19938,7 @@
       <c r="A12" s="47" t="n"/>
       <c r="B12" s="81" t="inlineStr">
         <is>
-          <t>INTERIORES (galeria y living)</t>
+          <t>INTERIORES (SE, galeria y living)</t>
         </is>
       </c>
       <c r="C12" s="18" t="inlineStr">
@@ -19961,7 +19961,7 @@
       <c r="A13" s="50" t="n"/>
       <c r="B13" s="82" t="inlineStr">
         <is>
-          <t>INTERIORES (deposito y lavadero)</t>
+          <t>INTERIORES (NE, deposito y lavadero)</t>
         </is>
       </c>
       <c r="C13" s="18" t="inlineStr">
@@ -20519,7 +20519,7 @@
       <c r="A43" s="47" t="n"/>
       <c r="B43" s="81" t="inlineStr">
         <is>
-          <t>INTERIORES (galeria, con la PV01)</t>
+          <t>INTERIORES (NO, galeria, con la PV01)</t>
         </is>
       </c>
       <c r="C43" s="18" t="inlineStr">
@@ -21091,7 +21091,7 @@
       <c r="A73" s="47" t="n"/>
       <c r="B73" s="81" t="inlineStr">
         <is>
-          <t>INTERIORES (vestidor)</t>
+          <t>INTERIORES (NE, vestidor)</t>
         </is>
       </c>
       <c r="C73" s="18" t="inlineStr">
@@ -21114,7 +21114,7 @@
       <c r="A74" s="50" t="n"/>
       <c r="B74" s="82" t="inlineStr">
         <is>
-          <t>INTERIORES (living comedor)</t>
+          <t>INTERIORES (NO, living comedor)</t>
         </is>
       </c>
       <c r="C74" s="18" t="inlineStr">
@@ -22145,7 +22145,7 @@
       <c r="A129" s="43" t="n"/>
       <c r="B129" s="79" t="inlineStr">
         <is>
-          <t>AISLADAS</t>
+          <t>AISLADAS (NE)</t>
         </is>
       </c>
       <c r="C129" s="18" t="inlineStr">
@@ -22191,7 +22191,7 @@
       <c r="A131" s="47" t="n"/>
       <c r="B131" s="81" t="inlineStr">
         <is>
-          <t>INTERIORES</t>
+          <t>INTERIORES (SO)</t>
         </is>
       </c>
       <c r="C131" s="18" t="inlineStr">
@@ -23268,7 +23268,7 @@
       <c r="A188" s="47" t="n"/>
       <c r="B188" s="81" t="inlineStr">
         <is>
-          <t>INTERIORES</t>
+          <t>INTERIORES (SO)</t>
         </is>
       </c>
       <c r="C188" s="18" t="inlineStr">
@@ -24957,7 +24957,7 @@
       <c r="A279" s="47" t="n"/>
       <c r="B279" s="81" t="inlineStr">
         <is>
-          <t>INTERIORES</t>
+          <t>INTERIORES (SE)</t>
         </is>
       </c>
       <c r="C279" s="18" t="inlineStr">
@@ -25506,7 +25506,7 @@
       <c r="A308" s="47" t="n"/>
       <c r="B308" s="81" t="inlineStr">
         <is>
-          <t>INTERIORES</t>
+          <t>INTERIORES (NO)</t>
         </is>
       </c>
       <c r="C308" s="18" t="inlineStr">
@@ -26003,7 +26003,7 @@
       <c r="A335" s="43" t="n"/>
       <c r="B335" s="79" t="inlineStr">
         <is>
-          <t>AISLADAS</t>
+          <t>AISLADAS (NE)</t>
         </is>
       </c>
       <c r="C335" s="18" t="inlineStr">
@@ -26049,7 +26049,7 @@
       <c r="A337" s="47" t="n"/>
       <c r="B337" s="81" t="inlineStr">
         <is>
-          <t>INTERIORES</t>
+          <t>INTERIORES (SO)</t>
         </is>
       </c>
       <c r="C337" s="18" t="inlineStr">

</xml_diff>

<commit_message>
Play room: el segundo 4,08 es la baranda de la escalera, no un muro; se saca el (2) de las aberturas
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01NNMcFTBbEuLfDho1wCZzu7
</commit_message>
<xml_diff>
--- a/planillas/planillas_estructura (para AutoCAD).xlsx
+++ b/planillas/planillas_estructura (para AutoCAD).xlsx
@@ -19691,7 +19691,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:G358"/>
+  <dimension ref="A1:G357"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8.1" customWidth="1" min="1" max="1"/>
@@ -22586,7 +22586,7 @@
       <c r="A152" s="43" t="n"/>
       <c r="B152" s="79" t="inlineStr">
         <is>
-          <t>VA01 (2)</t>
+          <t>VA01</t>
         </is>
       </c>
       <c r="C152" s="18" t="inlineStr">
@@ -24856,7 +24856,7 @@
       <c r="A274" s="90" t="n"/>
       <c r="B274" s="91" t="inlineStr">
         <is>
-          <t>VA04 (2)</t>
+          <t>VA04</t>
         </is>
       </c>
       <c r="C274" s="18" t="inlineStr">
@@ -24934,7 +24934,7 @@
       <c r="A278" s="47" t="n"/>
       <c r="B278" s="81" t="inlineStr">
         <is>
-          <t>INTERIORES</t>
+          <t>INTERIORES (NE)</t>
         </is>
       </c>
       <c r="C278" s="18" t="inlineStr">
@@ -24954,8 +24954,8 @@
       <c r="G278" s="53" t="n"/>
     </row>
     <row r="279" ht="19.8" customHeight="1">
-      <c r="A279" s="47" t="n"/>
-      <c r="B279" s="81" t="inlineStr">
+      <c r="A279" s="50" t="n"/>
+      <c r="B279" s="82" t="inlineStr">
         <is>
           <t>INTERIORES (SE)</t>
         </is>
@@ -24977,329 +24977,321 @@
       <c r="G279" s="53" t="n"/>
     </row>
     <row r="280" ht="19.8" customHeight="1">
-      <c r="A280" s="50" t="n"/>
-      <c r="B280" s="82" t="inlineStr">
-        <is>
-          <t>INTERIORES</t>
-        </is>
-      </c>
-      <c r="C280" s="18" t="inlineStr">
-        <is>
-          <t>4.08 x 3.00</t>
-        </is>
-      </c>
-      <c r="D280" s="19" t="n">
-        <v>12.24</v>
-      </c>
-      <c r="E280" s="59" t="n">
-        <v>25</v>
-      </c>
-      <c r="F280" s="80" t="n">
-        <v>306</v>
-      </c>
+      <c r="A280" s="36" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="B280" s="78" t="inlineStr">
+        <is>
+          <t>TECHOS O CIELORRASOS</t>
+        </is>
+      </c>
+      <c r="C280" s="47" t="n"/>
+      <c r="D280" s="18" t="n"/>
+      <c r="E280" s="18" t="n"/>
+      <c r="F280" s="20" t="n"/>
       <c r="G280" s="53" t="n"/>
     </row>
     <row r="281" ht="19.8" customHeight="1">
-      <c r="A281" s="36" t="inlineStr">
-        <is>
-          <t>3</t>
-        </is>
-      </c>
-      <c r="B281" s="78" t="inlineStr">
-        <is>
-          <t>TECHOS O CIELORRASOS</t>
-        </is>
-      </c>
-      <c r="C281" s="47" t="n"/>
-      <c r="D281" s="18" t="n"/>
-      <c r="E281" s="18" t="n"/>
-      <c r="F281" s="20" t="n"/>
+      <c r="A281" s="43" t="n"/>
+      <c r="B281" s="79" t="inlineStr">
+        <is>
+          <t>TECHO NO AISLADO</t>
+        </is>
+      </c>
+      <c r="C281" s="18" t="n"/>
+      <c r="D281" s="19" t="n"/>
+      <c r="E281" s="59" t="n">
+        <v>30</v>
+      </c>
+      <c r="F281" s="80" t="n"/>
       <c r="G281" s="53" t="n"/>
     </row>
     <row r="282" ht="19.8" customHeight="1">
-      <c r="A282" s="43" t="n"/>
-      <c r="B282" s="79" t="inlineStr">
-        <is>
-          <t>TECHO NO AISLADO</t>
-        </is>
-      </c>
-      <c r="C282" s="18" t="n"/>
-      <c r="D282" s="19" t="n"/>
+      <c r="A282" s="47" t="n"/>
+      <c r="B282" s="81" t="inlineStr">
+        <is>
+          <t>TECHO AISLADO</t>
+        </is>
+      </c>
+      <c r="C282" s="18" t="inlineStr">
+        <is>
+          <t>por croquis</t>
+        </is>
+      </c>
+      <c r="D282" s="19" t="n">
+        <v>16.85</v>
+      </c>
       <c r="E282" s="59" t="n">
-        <v>30</v>
-      </c>
-      <c r="F282" s="80" t="n"/>
+        <v>20</v>
+      </c>
+      <c r="F282" s="80" t="n">
+        <v>337</v>
+      </c>
       <c r="G282" s="53" t="n"/>
     </row>
     <row r="283" ht="19.8" customHeight="1">
-      <c r="A283" s="47" t="n"/>
-      <c r="B283" s="81" t="inlineStr">
-        <is>
-          <t>TECHO AISLADO</t>
-        </is>
-      </c>
-      <c r="C283" s="18" t="inlineStr">
+      <c r="A283" s="50" t="n"/>
+      <c r="B283" s="82" t="inlineStr">
+        <is>
+          <t>TECHO ENTREPISO</t>
+        </is>
+      </c>
+      <c r="C283" s="18" t="n"/>
+      <c r="D283" s="19" t="n"/>
+      <c r="E283" s="59" t="n">
+        <v>15</v>
+      </c>
+      <c r="F283" s="80" t="n"/>
+      <c r="G283" s="53" t="n"/>
+    </row>
+    <row r="284" ht="19.8" customHeight="1">
+      <c r="A284" s="36" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="B284" s="78" t="inlineStr">
+        <is>
+          <t>PISO</t>
+        </is>
+      </c>
+      <c r="C284" s="47" t="n"/>
+      <c r="D284" s="18" t="n"/>
+      <c r="E284" s="18" t="n"/>
+      <c r="F284" s="20" t="n"/>
+      <c r="G284" s="53" t="n"/>
+    </row>
+    <row r="285" ht="19.8" customHeight="1">
+      <c r="A285" s="43" t="n"/>
+      <c r="B285" s="79" t="inlineStr">
+        <is>
+          <t>SOBRE TIERRA</t>
+        </is>
+      </c>
+      <c r="C285" s="18" t="n"/>
+      <c r="D285" s="19" t="n"/>
+      <c r="E285" s="59" t="n">
+        <v>10</v>
+      </c>
+      <c r="F285" s="80" t="n"/>
+      <c r="G285" s="53" t="n"/>
+    </row>
+    <row r="286" ht="19.8" customHeight="1">
+      <c r="A286" s="50" t="n"/>
+      <c r="B286" s="82" t="inlineStr">
+        <is>
+          <t>SOBRE LOCAL OCUPADO</t>
+        </is>
+      </c>
+      <c r="C286" s="18" t="inlineStr">
         <is>
           <t>por croquis</t>
         </is>
       </c>
-      <c r="D283" s="19" t="n">
+      <c r="D286" s="24" t="n">
         <v>16.85</v>
       </c>
-      <c r="E283" s="59" t="n">
-        <v>20</v>
-      </c>
-      <c r="F283" s="80" t="n">
-        <v>337</v>
-      </c>
-      <c r="G283" s="53" t="n"/>
-    </row>
-    <row r="284" ht="19.8" customHeight="1">
-      <c r="A284" s="50" t="n"/>
-      <c r="B284" s="82" t="inlineStr">
-        <is>
-          <t>TECHO ENTREPISO</t>
-        </is>
-      </c>
-      <c r="C284" s="18" t="n"/>
-      <c r="D284" s="19" t="n"/>
-      <c r="E284" s="59" t="n">
+      <c r="E286" s="59" t="n">
         <v>15</v>
       </c>
-      <c r="F284" s="80" t="n"/>
-      <c r="G284" s="53" t="n"/>
-    </row>
-    <row r="285" ht="19.8" customHeight="1">
-      <c r="A285" s="36" t="inlineStr">
-        <is>
-          <t>4</t>
-        </is>
-      </c>
-      <c r="B285" s="78" t="inlineStr">
-        <is>
-          <t>PISO</t>
-        </is>
-      </c>
-      <c r="C285" s="47" t="n"/>
-      <c r="D285" s="18" t="n"/>
-      <c r="E285" s="18" t="n"/>
-      <c r="F285" s="20" t="n"/>
-      <c r="G285" s="53" t="n"/>
-    </row>
-    <row r="286" ht="19.8" customHeight="1">
-      <c r="A286" s="43" t="n"/>
-      <c r="B286" s="79" t="inlineStr">
-        <is>
-          <t>SOBRE TIERRA</t>
-        </is>
-      </c>
-      <c r="C286" s="18" t="n"/>
-      <c r="D286" s="19" t="n"/>
-      <c r="E286" s="59" t="n">
-        <v>10</v>
-      </c>
-      <c r="F286" s="80" t="n"/>
+      <c r="F286" s="80" t="n">
+        <v>252.8</v>
+      </c>
       <c r="G286" s="53" t="n"/>
     </row>
     <row r="287" ht="19.8" customHeight="1">
-      <c r="A287" s="50" t="n"/>
-      <c r="B287" s="82" t="inlineStr">
-        <is>
-          <t>SOBRE LOCAL OCUPADO</t>
-        </is>
-      </c>
-      <c r="C287" s="18" t="inlineStr">
-        <is>
-          <t>por croquis</t>
-        </is>
-      </c>
-      <c r="D287" s="24" t="n">
-        <v>16.85</v>
-      </c>
-      <c r="E287" s="59" t="n">
-        <v>15</v>
-      </c>
-      <c r="F287" s="80" t="n">
-        <v>252.8</v>
-      </c>
+      <c r="A287" s="36" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="B287" s="78" t="inlineStr">
+        <is>
+          <t>INFILTRACION</t>
+        </is>
+      </c>
+      <c r="C287" s="83" t="n"/>
+      <c r="D287" s="36" t="inlineStr">
+        <is>
+          <t>VOLUMEN (m3)</t>
+        </is>
+      </c>
+      <c r="E287" s="47" t="n"/>
+      <c r="F287" s="20" t="n"/>
       <c r="G287" s="53" t="n"/>
     </row>
     <row r="288" ht="19.8" customHeight="1">
-      <c r="A288" s="36" t="inlineStr">
-        <is>
-          <t>5</t>
-        </is>
-      </c>
-      <c r="B288" s="78" t="inlineStr">
-        <is>
-          <t>INFILTRACION</t>
-        </is>
-      </c>
-      <c r="C288" s="83" t="n"/>
-      <c r="D288" s="36" t="inlineStr">
-        <is>
-          <t>VOLUMEN (m3)</t>
-        </is>
-      </c>
-      <c r="E288" s="47" t="n"/>
-      <c r="F288" s="20" t="n"/>
+      <c r="A288" s="43" t="n"/>
+      <c r="B288" s="79" t="inlineStr">
+        <is>
+          <t>UNA PARED EXTERIOR</t>
+        </is>
+      </c>
+      <c r="C288" s="18" t="inlineStr">
+        <is>
+          <t>16.85 m2 x 3.00</t>
+        </is>
+      </c>
+      <c r="D288" s="22" t="n">
+        <v>50.55</v>
+      </c>
+      <c r="E288" s="59" t="n">
+        <v>6</v>
+      </c>
+      <c r="F288" s="80" t="n">
+        <v>303.3</v>
+      </c>
       <c r="G288" s="53" t="n"/>
     </row>
     <row r="289" ht="19.8" customHeight="1">
-      <c r="A289" s="43" t="n"/>
-      <c r="B289" s="79" t="inlineStr">
-        <is>
-          <t>UNA PARED EXTERIOR</t>
-        </is>
-      </c>
-      <c r="C289" s="18" t="inlineStr">
-        <is>
-          <t>16.85 m2 x 3.00</t>
-        </is>
-      </c>
-      <c r="D289" s="22" t="n">
-        <v>50.55</v>
-      </c>
+      <c r="A289" s="47" t="n"/>
+      <c r="B289" s="81" t="inlineStr">
+        <is>
+          <t>DOS PAREDES EXTERIORES</t>
+        </is>
+      </c>
+      <c r="C289" s="18" t="n"/>
+      <c r="D289" s="19" t="n"/>
       <c r="E289" s="59" t="n">
-        <v>6</v>
-      </c>
-      <c r="F289" s="80" t="n">
-        <v>303.3</v>
-      </c>
+        <v>9</v>
+      </c>
+      <c r="F289" s="80" t="n"/>
       <c r="G289" s="53" t="n"/>
     </row>
     <row r="290" ht="19.8" customHeight="1">
-      <c r="A290" s="47" t="n"/>
-      <c r="B290" s="81" t="inlineStr">
-        <is>
-          <t>DOS PAREDES EXTERIORES</t>
+      <c r="A290" s="50" t="n"/>
+      <c r="B290" s="82" t="inlineStr">
+        <is>
+          <t>TRES O MAS PAREDES EXTERIORES</t>
         </is>
       </c>
       <c r="C290" s="18" t="n"/>
       <c r="D290" s="19" t="n"/>
       <c r="E290" s="59" t="n">
-        <v>9</v>
-      </c>
-      <c r="F290" s="80" t="n"/>
+        <v>12</v>
+      </c>
+      <c r="F290" s="84" t="n"/>
       <c r="G290" s="53" t="n"/>
     </row>
     <row r="291" ht="19.8" customHeight="1">
-      <c r="A291" s="50" t="n"/>
-      <c r="B291" s="82" t="inlineStr">
-        <is>
-          <t>TRES O MAS PAREDES EXTERIORES</t>
-        </is>
-      </c>
-      <c r="C291" s="18" t="n"/>
-      <c r="D291" s="19" t="n"/>
-      <c r="E291" s="59" t="n">
-        <v>12</v>
-      </c>
-      <c r="F291" s="84" t="n"/>
+      <c r="A291" s="36" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="B291" s="78" t="inlineStr">
+        <is>
+          <t>SUBTOTAL</t>
+        </is>
+      </c>
+      <c r="C291" s="47" t="n"/>
+      <c r="D291" s="18" t="n"/>
+      <c r="E291" s="20" t="n"/>
+      <c r="F291" s="85" t="n">
+        <v>2059.1</v>
+      </c>
       <c r="G291" s="53" t="n"/>
     </row>
     <row r="292" ht="19.8" customHeight="1">
       <c r="A292" s="36" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B292" s="78" t="inlineStr">
         <is>
-          <t>SUBTOTAL</t>
-        </is>
-      </c>
-      <c r="C292" s="47" t="n"/>
-      <c r="D292" s="18" t="n"/>
-      <c r="E292" s="20" t="n"/>
+          <t>PERDIDA TOTAL</t>
+        </is>
+      </c>
+      <c r="C292" s="47" t="inlineStr">
+        <is>
+          <t>2059.10  X  1.07 (FI)  X  1 (FO)  X  1 (FZ)</t>
+        </is>
+      </c>
+      <c r="D292" s="12" t="n"/>
+      <c r="E292" s="14" t="n"/>
       <c r="F292" s="85" t="n">
-        <v>2365.1</v>
+        <v>2203.2</v>
       </c>
       <c r="G292" s="53" t="n"/>
     </row>
     <row r="293" ht="19.8" customHeight="1">
-      <c r="A293" s="36" t="inlineStr">
-        <is>
-          <t>7</t>
-        </is>
-      </c>
-      <c r="B293" s="78" t="inlineStr">
-        <is>
-          <t>PERDIDA TOTAL</t>
-        </is>
-      </c>
-      <c r="C293" s="47" t="inlineStr">
-        <is>
-          <t>2365.10  X  1.07 (FI)  X  1 (FO)  X  1 (FZ)</t>
+      <c r="A293" s="43" t="n"/>
+      <c r="B293" s="86" t="inlineStr">
+        <is>
+          <t>Carga de locales sin emisor</t>
+        </is>
+      </c>
+      <c r="C293" s="18" t="inlineStr">
+        <is>
+          <t>Escalera</t>
         </is>
       </c>
       <c r="D293" s="12" t="n"/>
-      <c r="E293" s="14" t="n"/>
-      <c r="F293" s="85" t="n">
-        <v>2530.7</v>
+      <c r="E293" s="39" t="n"/>
+      <c r="F293" s="87" t="n">
+        <v>1348.3</v>
       </c>
       <c r="G293" s="53" t="n"/>
     </row>
     <row r="294" ht="19.8" customHeight="1">
-      <c r="A294" s="43" t="n"/>
-      <c r="B294" s="86" t="inlineStr">
-        <is>
-          <t>Carga de locales sin emisor</t>
-        </is>
-      </c>
-      <c r="C294" s="18" t="inlineStr">
-        <is>
-          <t>Escalera</t>
-        </is>
-      </c>
+      <c r="A294" s="83" t="n"/>
+      <c r="B294" s="78" t="inlineStr">
+        <is>
+          <t>CARGA TOTAL A CUBRIR</t>
+        </is>
+      </c>
+      <c r="C294" s="47" t="n"/>
       <c r="D294" s="12" t="n"/>
-      <c r="E294" s="39" t="n"/>
-      <c r="F294" s="87" t="n">
-        <v>1348.3</v>
+      <c r="E294" s="14" t="n"/>
+      <c r="F294" s="85" t="n">
+        <v>3551.5</v>
       </c>
       <c r="G294" s="53" t="n"/>
     </row>
     <row r="295" ht="19.8" customHeight="1">
-      <c r="A295" s="83" t="n"/>
-      <c r="B295" s="78" t="inlineStr">
-        <is>
-          <t>CARGA TOTAL A CUBRIR</t>
-        </is>
-      </c>
-      <c r="C295" s="47" t="n"/>
+      <c r="A295" s="47" t="n"/>
+      <c r="B295" s="88" t="inlineStr">
+        <is>
+          <t>Salto termico:  dt = (te+ts)/2 - ti</t>
+        </is>
+      </c>
+      <c r="C295" s="18" t="inlineStr">
+        <is>
+          <t>86 - 20 = 66 C</t>
+        </is>
+      </c>
       <c r="D295" s="12" t="n"/>
-      <c r="E295" s="14" t="n"/>
-      <c r="F295" s="85" t="n">
-        <v>3879</v>
-      </c>
+      <c r="E295" s="39" t="n"/>
+      <c r="F295" s="61" t="n"/>
       <c r="G295" s="53" t="n"/>
     </row>
     <row r="296" ht="19.8" customHeight="1">
       <c r="A296" s="47" t="n"/>
-      <c r="B296" s="88" t="inlineStr">
-        <is>
-          <t>Salto termico:  dt = (te+ts)/2 - ti</t>
-        </is>
-      </c>
-      <c r="C296" s="18" t="inlineStr">
-        <is>
-          <t>86 - 20 = 66 C</t>
-        </is>
+      <c r="B296" s="60" t="inlineStr">
+        <is>
+          <t>Kcal/h por elemento</t>
+        </is>
+      </c>
+      <c r="C296" s="19" t="n">
+        <v>274.4</v>
       </c>
       <c r="D296" s="12" t="n"/>
       <c r="E296" s="39" t="n"/>
-      <c r="F296" s="61" t="n"/>
+      <c r="F296" s="20" t="n"/>
       <c r="G296" s="53" t="n"/>
     </row>
     <row r="297" ht="19.8" customHeight="1">
       <c r="A297" s="47" t="n"/>
       <c r="B297" s="60" t="inlineStr">
         <is>
-          <t>Kcal/h por elemento</t>
-        </is>
-      </c>
-      <c r="C297" s="19" t="n">
-        <v>274.4</v>
+          <t>Elementos necesarios</t>
+        </is>
+      </c>
+      <c r="C297" s="59" t="n">
+        <v>13</v>
       </c>
       <c r="D297" s="12" t="n"/>
       <c r="E297" s="39" t="n"/>
@@ -25310,11 +25302,11 @@
       <c r="A298" s="47" t="n"/>
       <c r="B298" s="60" t="inlineStr">
         <is>
-          <t>Elementos necesarios</t>
+          <t>Ancho del radiador (cm)</t>
         </is>
       </c>
       <c r="C298" s="59" t="n">
-        <v>15</v>
+        <v>104</v>
       </c>
       <c r="D298" s="12" t="n"/>
       <c r="E298" s="39" t="n"/>
@@ -25322,14 +25314,16 @@
       <c r="G298" s="53" t="n"/>
     </row>
     <row r="299" ht="19.8" customHeight="1">
-      <c r="A299" s="47" t="n"/>
+      <c r="A299" s="50" t="n"/>
       <c r="B299" s="60" t="inlineStr">
         <is>
-          <t>Ancho del radiador (cm)</t>
-        </is>
-      </c>
-      <c r="C299" s="59" t="n">
-        <v>120</v>
+          <t>Radiador adoptado</t>
+        </is>
+      </c>
+      <c r="C299" s="18" t="inlineStr">
+        <is>
+          <t>Peisa Tropical 80-500</t>
+        </is>
       </c>
       <c r="D299" s="12" t="n"/>
       <c r="E299" s="39" t="n"/>
@@ -25337,145 +25331,151 @@
       <c r="G299" s="53" t="n"/>
     </row>
     <row r="300" ht="19.8" customHeight="1">
-      <c r="A300" s="50" t="n"/>
-      <c r="B300" s="60" t="inlineStr">
-        <is>
-          <t>Radiador adoptado</t>
-        </is>
-      </c>
-      <c r="C300" s="18" t="inlineStr">
-        <is>
-          <t>Peisa Tropical 80-500</t>
-        </is>
-      </c>
-      <c r="D300" s="12" t="n"/>
-      <c r="E300" s="39" t="n"/>
-      <c r="F300" s="20" t="n"/>
+      <c r="A300" s="8" t="inlineStr">
+        <is>
+          <t>LOCAL  15 - Dormitorio Sur   (PA)   -   altura 3.00 m</t>
+        </is>
+      </c>
+      <c r="B300" s="11" t="n"/>
+      <c r="C300" s="11" t="n"/>
+      <c r="D300" s="11" t="n"/>
+      <c r="E300" s="11" t="n"/>
+      <c r="F300" s="42" t="n"/>
       <c r="G300" s="53" t="n"/>
     </row>
-    <row r="301" ht="19.8" customHeight="1">
-      <c r="A301" s="8" t="inlineStr">
-        <is>
-          <t>LOCAL  15 - Dormitorio Sur   (PA)   -   altura 3.00 m</t>
-        </is>
-      </c>
-      <c r="B301" s="11" t="n"/>
-      <c r="C301" s="11" t="n"/>
-      <c r="D301" s="11" t="n"/>
-      <c r="E301" s="11" t="n"/>
-      <c r="F301" s="42" t="n"/>
+    <row r="301" ht="32" customHeight="1">
+      <c r="A301" s="2" t="inlineStr">
+        <is>
+          <t>Nro</t>
+        </is>
+      </c>
+      <c r="B301" s="2" t="inlineStr">
+        <is>
+          <t>DESCRIPCION</t>
+        </is>
+      </c>
+      <c r="C301" s="2" t="inlineStr">
+        <is>
+          <t>DIMENSIONES (m)</t>
+        </is>
+      </c>
+      <c r="D301" s="2" t="inlineStr">
+        <is>
+          <t>AREA (m2)</t>
+        </is>
+      </c>
+      <c r="E301" s="2" t="inlineStr">
+        <is>
+          <t>FACTOR</t>
+        </is>
+      </c>
+      <c r="F301" s="2" t="inlineStr">
+        <is>
+          <t>PERDIDA CALOR (Kcal/h)</t>
+        </is>
+      </c>
       <c r="G301" s="53" t="n"/>
     </row>
-    <row r="302" ht="32" customHeight="1">
-      <c r="A302" s="2" t="inlineStr">
-        <is>
-          <t>Nro</t>
-        </is>
-      </c>
-      <c r="B302" s="2" t="inlineStr">
-        <is>
-          <t>DESCRIPCION</t>
-        </is>
-      </c>
-      <c r="C302" s="2" t="inlineStr">
-        <is>
-          <t>DIMENSIONES (m)</t>
-        </is>
-      </c>
-      <c r="D302" s="2" t="inlineStr">
-        <is>
-          <t>AREA (m2)</t>
-        </is>
-      </c>
-      <c r="E302" s="2" t="inlineStr">
-        <is>
-          <t>FACTOR</t>
-        </is>
-      </c>
-      <c r="F302" s="2" t="inlineStr">
-        <is>
-          <t>PERDIDA CALOR (Kcal/h)</t>
-        </is>
-      </c>
+    <row r="302" ht="19.8" customHeight="1">
+      <c r="A302" s="36" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="B302" s="78" t="inlineStr">
+        <is>
+          <t>VENTANA</t>
+        </is>
+      </c>
+      <c r="C302" s="43" t="n"/>
+      <c r="D302" s="58" t="n"/>
+      <c r="E302" s="58" t="n"/>
+      <c r="F302" s="61" t="n"/>
       <c r="G302" s="53" t="n"/>
     </row>
     <row r="303" ht="19.8" customHeight="1">
-      <c r="A303" s="36" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="B303" s="78" t="inlineStr">
-        <is>
-          <t>VENTANA</t>
-        </is>
-      </c>
-      <c r="C303" s="43" t="n"/>
-      <c r="D303" s="58" t="n"/>
-      <c r="E303" s="58" t="n"/>
-      <c r="F303" s="61" t="n"/>
+      <c r="A303" s="90" t="n"/>
+      <c r="B303" s="91" t="inlineStr">
+        <is>
+          <t>PV04</t>
+        </is>
+      </c>
+      <c r="C303" s="18" t="inlineStr">
+        <is>
+          <t>2.06 x 3.00</t>
+        </is>
+      </c>
+      <c r="D303" s="19" t="n">
+        <v>6.18</v>
+      </c>
+      <c r="E303" s="59" t="n">
+        <v>60</v>
+      </c>
+      <c r="F303" s="80" t="n">
+        <v>370.8</v>
+      </c>
       <c r="G303" s="53" t="n"/>
     </row>
     <row r="304" ht="19.8" customHeight="1">
-      <c r="A304" s="90" t="n"/>
-      <c r="B304" s="91" t="inlineStr">
-        <is>
-          <t>PV04</t>
-        </is>
-      </c>
-      <c r="C304" s="18" t="inlineStr">
-        <is>
-          <t>2.06 x 3.00</t>
-        </is>
-      </c>
-      <c r="D304" s="19" t="n">
-        <v>6.18</v>
-      </c>
-      <c r="E304" s="59" t="n">
-        <v>60</v>
-      </c>
-      <c r="F304" s="80" t="n">
-        <v>370.8</v>
-      </c>
+      <c r="A304" s="36" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="B304" s="78" t="inlineStr">
+        <is>
+          <t>PAREDES EXTERIORES</t>
+        </is>
+      </c>
+      <c r="C304" s="47" t="n"/>
+      <c r="D304" s="18" t="n"/>
+      <c r="E304" s="18" t="n"/>
+      <c r="F304" s="20" t="n"/>
       <c r="G304" s="53" t="n"/>
     </row>
     <row r="305" ht="19.8" customHeight="1">
-      <c r="A305" s="36" t="inlineStr">
-        <is>
-          <t>2</t>
-        </is>
-      </c>
-      <c r="B305" s="78" t="inlineStr">
-        <is>
-          <t>PAREDES EXTERIORES</t>
-        </is>
-      </c>
-      <c r="C305" s="47" t="n"/>
-      <c r="D305" s="18" t="n"/>
-      <c r="E305" s="18" t="n"/>
-      <c r="F305" s="20" t="n"/>
+      <c r="A305" s="43" t="n"/>
+      <c r="B305" s="79" t="inlineStr">
+        <is>
+          <t>AISLADAS (SE)</t>
+        </is>
+      </c>
+      <c r="C305" s="18" t="inlineStr">
+        <is>
+          <t>4.05 x 3.00</t>
+        </is>
+      </c>
+      <c r="D305" s="19" t="n">
+        <v>12.15</v>
+      </c>
+      <c r="E305" s="59" t="n">
+        <v>20</v>
+      </c>
+      <c r="F305" s="80" t="n">
+        <v>243</v>
+      </c>
       <c r="G305" s="53" t="n"/>
     </row>
     <row r="306" ht="19.8" customHeight="1">
-      <c r="A306" s="43" t="n"/>
-      <c r="B306" s="79" t="inlineStr">
-        <is>
-          <t>AISLADAS (SE)</t>
+      <c r="A306" s="47" t="n"/>
+      <c r="B306" s="81" t="inlineStr">
+        <is>
+          <t>AISLADAS</t>
         </is>
       </c>
       <c r="C306" s="18" t="inlineStr">
         <is>
-          <t>4.05 x 3.00</t>
+          <t>3.50 x 3.00</t>
         </is>
       </c>
       <c r="D306" s="19" t="n">
-        <v>12.15</v>
+        <v>10.5</v>
       </c>
       <c r="E306" s="59" t="n">
         <v>20</v>
       </c>
       <c r="F306" s="80" t="n">
-        <v>243</v>
+        <v>210</v>
       </c>
       <c r="G306" s="53" t="n"/>
     </row>
@@ -25483,366 +25483,358 @@
       <c r="A307" s="47" t="n"/>
       <c r="B307" s="81" t="inlineStr">
         <is>
-          <t>AISLADAS</t>
+          <t>INTERIORES (NO)</t>
         </is>
       </c>
       <c r="C307" s="18" t="inlineStr">
         <is>
+          <t>4.05 x 3.00</t>
+        </is>
+      </c>
+      <c r="D307" s="19" t="n">
+        <v>12.15</v>
+      </c>
+      <c r="E307" s="59" t="n">
+        <v>25</v>
+      </c>
+      <c r="F307" s="80" t="n">
+        <v>303.8</v>
+      </c>
+      <c r="G307" s="53" t="n"/>
+    </row>
+    <row r="308" ht="19.8" customHeight="1">
+      <c r="A308" s="50" t="n"/>
+      <c r="B308" s="82" t="inlineStr">
+        <is>
+          <t>INTERIORES</t>
+        </is>
+      </c>
+      <c r="C308" s="18" t="inlineStr">
+        <is>
           <t>3.50 x 3.00</t>
         </is>
       </c>
-      <c r="D307" s="19" t="n">
+      <c r="D308" s="19" t="n">
         <v>10.5</v>
-      </c>
-      <c r="E307" s="59" t="n">
-        <v>20</v>
-      </c>
-      <c r="F307" s="80" t="n">
-        <v>210</v>
-      </c>
-      <c r="G307" s="53" t="n"/>
-    </row>
-    <row r="308" ht="19.8" customHeight="1">
-      <c r="A308" s="47" t="n"/>
-      <c r="B308" s="81" t="inlineStr">
-        <is>
-          <t>INTERIORES (NO)</t>
-        </is>
-      </c>
-      <c r="C308" s="18" t="inlineStr">
-        <is>
-          <t>4.05 x 3.00</t>
-        </is>
-      </c>
-      <c r="D308" s="19" t="n">
-        <v>12.15</v>
       </c>
       <c r="E308" s="59" t="n">
         <v>25</v>
       </c>
       <c r="F308" s="80" t="n">
-        <v>303.8</v>
+        <v>262.5</v>
       </c>
       <c r="G308" s="53" t="n"/>
     </row>
     <row r="309" ht="19.8" customHeight="1">
-      <c r="A309" s="50" t="n"/>
-      <c r="B309" s="82" t="inlineStr">
-        <is>
-          <t>INTERIORES</t>
-        </is>
-      </c>
-      <c r="C309" s="18" t="inlineStr">
-        <is>
-          <t>3.50 x 3.00</t>
-        </is>
-      </c>
-      <c r="D309" s="19" t="n">
-        <v>10.5</v>
-      </c>
-      <c r="E309" s="59" t="n">
-        <v>25</v>
-      </c>
-      <c r="F309" s="80" t="n">
-        <v>262.5</v>
-      </c>
+      <c r="A309" s="36" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="B309" s="78" t="inlineStr">
+        <is>
+          <t>TECHOS O CIELORRASOS</t>
+        </is>
+      </c>
+      <c r="C309" s="47" t="n"/>
+      <c r="D309" s="18" t="n"/>
+      <c r="E309" s="18" t="n"/>
+      <c r="F309" s="20" t="n"/>
       <c r="G309" s="53" t="n"/>
     </row>
     <row r="310" ht="19.8" customHeight="1">
-      <c r="A310" s="36" t="inlineStr">
-        <is>
-          <t>3</t>
-        </is>
-      </c>
-      <c r="B310" s="78" t="inlineStr">
-        <is>
-          <t>TECHOS O CIELORRASOS</t>
-        </is>
-      </c>
-      <c r="C310" s="47" t="n"/>
-      <c r="D310" s="18" t="n"/>
-      <c r="E310" s="18" t="n"/>
-      <c r="F310" s="20" t="n"/>
+      <c r="A310" s="43" t="n"/>
+      <c r="B310" s="79" t="inlineStr">
+        <is>
+          <t>TECHO NO AISLADO</t>
+        </is>
+      </c>
+      <c r="C310" s="18" t="n"/>
+      <c r="D310" s="19" t="n"/>
+      <c r="E310" s="59" t="n">
+        <v>30</v>
+      </c>
+      <c r="F310" s="80" t="n"/>
       <c r="G310" s="53" t="n"/>
     </row>
     <row r="311" ht="19.8" customHeight="1">
-      <c r="A311" s="43" t="n"/>
-      <c r="B311" s="79" t="inlineStr">
-        <is>
-          <t>TECHO NO AISLADO</t>
-        </is>
-      </c>
-      <c r="C311" s="18" t="n"/>
-      <c r="D311" s="19" t="n"/>
+      <c r="A311" s="47" t="n"/>
+      <c r="B311" s="81" t="inlineStr">
+        <is>
+          <t>TECHO AISLADO</t>
+        </is>
+      </c>
+      <c r="C311" s="18" t="inlineStr">
+        <is>
+          <t>por croquis</t>
+        </is>
+      </c>
+      <c r="D311" s="19" t="n">
+        <v>14.17</v>
+      </c>
       <c r="E311" s="59" t="n">
-        <v>30</v>
-      </c>
-      <c r="F311" s="80" t="n"/>
+        <v>20</v>
+      </c>
+      <c r="F311" s="80" t="n">
+        <v>283.4</v>
+      </c>
       <c r="G311" s="53" t="n"/>
     </row>
     <row r="312" ht="19.8" customHeight="1">
-      <c r="A312" s="47" t="n"/>
-      <c r="B312" s="81" t="inlineStr">
-        <is>
-          <t>TECHO AISLADO</t>
-        </is>
-      </c>
-      <c r="C312" s="18" t="inlineStr">
+      <c r="A312" s="50" t="n"/>
+      <c r="B312" s="82" t="inlineStr">
+        <is>
+          <t>TECHO ENTREPISO</t>
+        </is>
+      </c>
+      <c r="C312" s="18" t="n"/>
+      <c r="D312" s="19" t="n"/>
+      <c r="E312" s="59" t="n">
+        <v>15</v>
+      </c>
+      <c r="F312" s="80" t="n"/>
+      <c r="G312" s="53" t="n"/>
+    </row>
+    <row r="313" ht="19.8" customHeight="1">
+      <c r="A313" s="36" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="B313" s="78" t="inlineStr">
+        <is>
+          <t>PISO</t>
+        </is>
+      </c>
+      <c r="C313" s="47" t="n"/>
+      <c r="D313" s="18" t="n"/>
+      <c r="E313" s="18" t="n"/>
+      <c r="F313" s="20" t="n"/>
+      <c r="G313" s="53" t="n"/>
+    </row>
+    <row r="314" ht="19.8" customHeight="1">
+      <c r="A314" s="43" t="n"/>
+      <c r="B314" s="79" t="inlineStr">
+        <is>
+          <t>SOBRE TIERRA</t>
+        </is>
+      </c>
+      <c r="C314" s="18" t="n"/>
+      <c r="D314" s="19" t="n"/>
+      <c r="E314" s="59" t="n">
+        <v>10</v>
+      </c>
+      <c r="F314" s="80" t="n"/>
+      <c r="G314" s="53" t="n"/>
+    </row>
+    <row r="315" ht="19.8" customHeight="1">
+      <c r="A315" s="50" t="n"/>
+      <c r="B315" s="82" t="inlineStr">
+        <is>
+          <t>SOBRE LOCAL OCUPADO</t>
+        </is>
+      </c>
+      <c r="C315" s="18" t="inlineStr">
         <is>
           <t>por croquis</t>
         </is>
       </c>
-      <c r="D312" s="19" t="n">
+      <c r="D315" s="24" t="n">
         <v>14.17</v>
       </c>
-      <c r="E312" s="59" t="n">
-        <v>20</v>
-      </c>
-      <c r="F312" s="80" t="n">
-        <v>283.4</v>
-      </c>
-      <c r="G312" s="53" t="n"/>
-    </row>
-    <row r="313" ht="19.8" customHeight="1">
-      <c r="A313" s="50" t="n"/>
-      <c r="B313" s="82" t="inlineStr">
-        <is>
-          <t>TECHO ENTREPISO</t>
-        </is>
-      </c>
-      <c r="C313" s="18" t="n"/>
-      <c r="D313" s="19" t="n"/>
-      <c r="E313" s="59" t="n">
+      <c r="E315" s="59" t="n">
         <v>15</v>
       </c>
-      <c r="F313" s="80" t="n"/>
-      <c r="G313" s="53" t="n"/>
-    </row>
-    <row r="314" ht="19.8" customHeight="1">
-      <c r="A314" s="36" t="inlineStr">
-        <is>
-          <t>4</t>
-        </is>
-      </c>
-      <c r="B314" s="78" t="inlineStr">
-        <is>
-          <t>PISO</t>
-        </is>
-      </c>
-      <c r="C314" s="47" t="n"/>
-      <c r="D314" s="18" t="n"/>
-      <c r="E314" s="18" t="n"/>
-      <c r="F314" s="20" t="n"/>
-      <c r="G314" s="53" t="n"/>
-    </row>
-    <row r="315" ht="19.8" customHeight="1">
-      <c r="A315" s="43" t="n"/>
-      <c r="B315" s="79" t="inlineStr">
-        <is>
-          <t>SOBRE TIERRA</t>
-        </is>
-      </c>
-      <c r="C315" s="18" t="n"/>
-      <c r="D315" s="19" t="n"/>
-      <c r="E315" s="59" t="n">
-        <v>10</v>
-      </c>
-      <c r="F315" s="80" t="n"/>
+      <c r="F315" s="80" t="n">
+        <v>212.6</v>
+      </c>
       <c r="G315" s="53" t="n"/>
     </row>
     <row r="316" ht="19.8" customHeight="1">
-      <c r="A316" s="50" t="n"/>
-      <c r="B316" s="82" t="inlineStr">
-        <is>
-          <t>SOBRE LOCAL OCUPADO</t>
-        </is>
-      </c>
-      <c r="C316" s="18" t="inlineStr">
-        <is>
-          <t>por croquis</t>
-        </is>
-      </c>
-      <c r="D316" s="24" t="n">
-        <v>14.17</v>
-      </c>
-      <c r="E316" s="59" t="n">
-        <v>15</v>
-      </c>
-      <c r="F316" s="80" t="n">
-        <v>212.6</v>
-      </c>
+      <c r="A316" s="36" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="B316" s="78" t="inlineStr">
+        <is>
+          <t>INFILTRACION</t>
+        </is>
+      </c>
+      <c r="C316" s="83" t="n"/>
+      <c r="D316" s="36" t="inlineStr">
+        <is>
+          <t>VOLUMEN (m3)</t>
+        </is>
+      </c>
+      <c r="E316" s="47" t="n"/>
+      <c r="F316" s="20" t="n"/>
       <c r="G316" s="53" t="n"/>
     </row>
     <row r="317" ht="19.8" customHeight="1">
-      <c r="A317" s="36" t="inlineStr">
-        <is>
-          <t>5</t>
-        </is>
-      </c>
-      <c r="B317" s="78" t="inlineStr">
-        <is>
-          <t>INFILTRACION</t>
-        </is>
-      </c>
-      <c r="C317" s="83" t="n"/>
-      <c r="D317" s="36" t="inlineStr">
-        <is>
-          <t>VOLUMEN (m3)</t>
-        </is>
-      </c>
-      <c r="E317" s="47" t="n"/>
-      <c r="F317" s="20" t="n"/>
+      <c r="A317" s="43" t="n"/>
+      <c r="B317" s="79" t="inlineStr">
+        <is>
+          <t>UNA PARED EXTERIOR</t>
+        </is>
+      </c>
+      <c r="C317" s="18" t="n"/>
+      <c r="D317" s="22" t="n"/>
+      <c r="E317" s="59" t="n">
+        <v>6</v>
+      </c>
+      <c r="F317" s="80" t="n"/>
       <c r="G317" s="53" t="n"/>
     </row>
     <row r="318" ht="19.8" customHeight="1">
-      <c r="A318" s="43" t="n"/>
-      <c r="B318" s="79" t="inlineStr">
-        <is>
-          <t>UNA PARED EXTERIOR</t>
-        </is>
-      </c>
-      <c r="C318" s="18" t="n"/>
-      <c r="D318" s="22" t="n"/>
+      <c r="A318" s="47" t="n"/>
+      <c r="B318" s="81" t="inlineStr">
+        <is>
+          <t>DOS PAREDES EXTERIORES</t>
+        </is>
+      </c>
+      <c r="C318" s="18" t="inlineStr">
+        <is>
+          <t>14.17 m2 x 3.00</t>
+        </is>
+      </c>
+      <c r="D318" s="19" t="n">
+        <v>42.51</v>
+      </c>
       <c r="E318" s="59" t="n">
-        <v>6</v>
-      </c>
-      <c r="F318" s="80" t="n"/>
+        <v>9</v>
+      </c>
+      <c r="F318" s="80" t="n">
+        <v>382.6</v>
+      </c>
       <c r="G318" s="53" t="n"/>
     </row>
     <row r="319" ht="19.8" customHeight="1">
-      <c r="A319" s="47" t="n"/>
-      <c r="B319" s="81" t="inlineStr">
-        <is>
-          <t>DOS PAREDES EXTERIORES</t>
-        </is>
-      </c>
-      <c r="C319" s="18" t="inlineStr">
-        <is>
-          <t>14.17 m2 x 3.00</t>
-        </is>
-      </c>
-      <c r="D319" s="19" t="n">
-        <v>42.51</v>
-      </c>
+      <c r="A319" s="50" t="n"/>
+      <c r="B319" s="82" t="inlineStr">
+        <is>
+          <t>TRES O MAS PAREDES EXTERIORES</t>
+        </is>
+      </c>
+      <c r="C319" s="18" t="n"/>
+      <c r="D319" s="19" t="n"/>
       <c r="E319" s="59" t="n">
-        <v>9</v>
-      </c>
-      <c r="F319" s="80" t="n">
-        <v>382.6</v>
-      </c>
+        <v>12</v>
+      </c>
+      <c r="F319" s="84" t="n"/>
       <c r="G319" s="53" t="n"/>
     </row>
     <row r="320" ht="19.8" customHeight="1">
-      <c r="A320" s="50" t="n"/>
-      <c r="B320" s="82" t="inlineStr">
-        <is>
-          <t>TRES O MAS PAREDES EXTERIORES</t>
-        </is>
-      </c>
-      <c r="C320" s="18" t="n"/>
-      <c r="D320" s="19" t="n"/>
-      <c r="E320" s="59" t="n">
-        <v>12</v>
-      </c>
-      <c r="F320" s="84" t="n"/>
+      <c r="A320" s="36" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="B320" s="78" t="inlineStr">
+        <is>
+          <t>SUBTOTAL</t>
+        </is>
+      </c>
+      <c r="C320" s="47" t="n"/>
+      <c r="D320" s="18" t="n"/>
+      <c r="E320" s="20" t="n"/>
+      <c r="F320" s="85" t="n">
+        <v>2268.7</v>
+      </c>
       <c r="G320" s="53" t="n"/>
     </row>
     <row r="321" ht="19.8" customHeight="1">
       <c r="A321" s="36" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B321" s="78" t="inlineStr">
         <is>
-          <t>SUBTOTAL</t>
-        </is>
-      </c>
-      <c r="C321" s="47" t="n"/>
-      <c r="D321" s="18" t="n"/>
-      <c r="E321" s="20" t="n"/>
+          <t>PERDIDA TOTAL</t>
+        </is>
+      </c>
+      <c r="C321" s="47" t="inlineStr">
+        <is>
+          <t>2268.70  X  1.07 (FI)  X  1 (FO)  X  1 (FZ)</t>
+        </is>
+      </c>
+      <c r="D321" s="12" t="n"/>
+      <c r="E321" s="14" t="n"/>
       <c r="F321" s="85" t="n">
-        <v>2268.7</v>
+        <v>2427.5</v>
       </c>
       <c r="G321" s="53" t="n"/>
     </row>
     <row r="322" ht="19.8" customHeight="1">
-      <c r="A322" s="36" t="inlineStr">
-        <is>
-          <t>7</t>
-        </is>
-      </c>
-      <c r="B322" s="78" t="inlineStr">
-        <is>
-          <t>PERDIDA TOTAL</t>
-        </is>
-      </c>
-      <c r="C322" s="47" t="inlineStr">
-        <is>
-          <t>2268.70  X  1.07 (FI)  X  1 (FO)  X  1 (FZ)</t>
-        </is>
-      </c>
+      <c r="A322" s="43" t="n"/>
+      <c r="B322" s="86" t="inlineStr">
+        <is>
+          <t>Carga de locales sin emisor</t>
+        </is>
+      </c>
+      <c r="C322" s="18" t="n"/>
       <c r="D322" s="12" t="n"/>
-      <c r="E322" s="14" t="n"/>
-      <c r="F322" s="85" t="n">
+      <c r="E322" s="39" t="n"/>
+      <c r="F322" s="87" t="n"/>
+      <c r="G322" s="53" t="n"/>
+    </row>
+    <row r="323" ht="19.8" customHeight="1">
+      <c r="A323" s="83" t="n"/>
+      <c r="B323" s="78" t="inlineStr">
+        <is>
+          <t>CARGA TOTAL A CUBRIR</t>
+        </is>
+      </c>
+      <c r="C323" s="47" t="n"/>
+      <c r="D323" s="12" t="n"/>
+      <c r="E323" s="14" t="n"/>
+      <c r="F323" s="85" t="n">
         <v>2427.5</v>
       </c>
-      <c r="G322" s="53" t="n"/>
-    </row>
-    <row r="323" ht="19.8" customHeight="1">
-      <c r="A323" s="43" t="n"/>
-      <c r="B323" s="86" t="inlineStr">
-        <is>
-          <t>Carga de locales sin emisor</t>
-        </is>
-      </c>
-      <c r="C323" s="18" t="n"/>
-      <c r="D323" s="12" t="n"/>
-      <c r="E323" s="39" t="n"/>
-      <c r="F323" s="87" t="n"/>
       <c r="G323" s="53" t="n"/>
     </row>
     <row r="324" ht="19.8" customHeight="1">
-      <c r="A324" s="83" t="n"/>
-      <c r="B324" s="78" t="inlineStr">
-        <is>
-          <t>CARGA TOTAL A CUBRIR</t>
-        </is>
-      </c>
-      <c r="C324" s="47" t="n"/>
+      <c r="A324" s="47" t="n"/>
+      <c r="B324" s="88" t="inlineStr">
+        <is>
+          <t>Salto termico:  dt = (te+ts)/2 - ti</t>
+        </is>
+      </c>
+      <c r="C324" s="18" t="inlineStr">
+        <is>
+          <t>86 - 20 = 66 C</t>
+        </is>
+      </c>
       <c r="D324" s="12" t="n"/>
-      <c r="E324" s="14" t="n"/>
-      <c r="F324" s="85" t="n">
-        <v>2427.5</v>
-      </c>
+      <c r="E324" s="39" t="n"/>
+      <c r="F324" s="61" t="n"/>
       <c r="G324" s="53" t="n"/>
     </row>
     <row r="325" ht="19.8" customHeight="1">
       <c r="A325" s="47" t="n"/>
-      <c r="B325" s="88" t="inlineStr">
-        <is>
-          <t>Salto termico:  dt = (te+ts)/2 - ti</t>
-        </is>
-      </c>
-      <c r="C325" s="18" t="inlineStr">
-        <is>
-          <t>86 - 20 = 66 C</t>
-        </is>
+      <c r="B325" s="60" t="inlineStr">
+        <is>
+          <t>Kcal/h por elemento</t>
+        </is>
+      </c>
+      <c r="C325" s="19" t="n">
+        <v>274.4</v>
       </c>
       <c r="D325" s="12" t="n"/>
       <c r="E325" s="39" t="n"/>
-      <c r="F325" s="61" t="n"/>
+      <c r="F325" s="20" t="n"/>
       <c r="G325" s="53" t="n"/>
     </row>
     <row r="326" ht="19.8" customHeight="1">
       <c r="A326" s="47" t="n"/>
       <c r="B326" s="60" t="inlineStr">
         <is>
-          <t>Kcal/h por elemento</t>
-        </is>
-      </c>
-      <c r="C326" s="19" t="n">
-        <v>274.4</v>
+          <t>Elementos necesarios</t>
+        </is>
+      </c>
+      <c r="C326" s="59" t="n">
+        <v>9</v>
       </c>
       <c r="D326" s="12" t="n"/>
       <c r="E326" s="39" t="n"/>
@@ -25853,11 +25845,11 @@
       <c r="A327" s="47" t="n"/>
       <c r="B327" s="60" t="inlineStr">
         <is>
-          <t>Elementos necesarios</t>
+          <t>Ancho del radiador (cm)</t>
         </is>
       </c>
       <c r="C327" s="59" t="n">
-        <v>9</v>
+        <v>72</v>
       </c>
       <c r="D327" s="12" t="n"/>
       <c r="E327" s="39" t="n"/>
@@ -25865,14 +25857,16 @@
       <c r="G327" s="53" t="n"/>
     </row>
     <row r="328" ht="19.8" customHeight="1">
-      <c r="A328" s="47" t="n"/>
+      <c r="A328" s="50" t="n"/>
       <c r="B328" s="60" t="inlineStr">
         <is>
-          <t>Ancho del radiador (cm)</t>
-        </is>
-      </c>
-      <c r="C328" s="59" t="n">
-        <v>72</v>
+          <t>Radiador adoptado</t>
+        </is>
+      </c>
+      <c r="C328" s="18" t="inlineStr">
+        <is>
+          <t>Peisa Tropical 80-500</t>
+        </is>
       </c>
       <c r="D328" s="12" t="n"/>
       <c r="E328" s="39" t="n"/>
@@ -25880,145 +25874,151 @@
       <c r="G328" s="53" t="n"/>
     </row>
     <row r="329" ht="19.8" customHeight="1">
-      <c r="A329" s="50" t="n"/>
-      <c r="B329" s="60" t="inlineStr">
-        <is>
-          <t>Radiador adoptado</t>
-        </is>
-      </c>
-      <c r="C329" s="18" t="inlineStr">
-        <is>
-          <t>Peisa Tropical 80-500</t>
-        </is>
-      </c>
-      <c r="D329" s="12" t="n"/>
-      <c r="E329" s="39" t="n"/>
-      <c r="F329" s="20" t="n"/>
+      <c r="A329" s="8" t="inlineStr">
+        <is>
+          <t>LOCAL  17 - Bano   (PA)   -   altura 3.00 m</t>
+        </is>
+      </c>
+      <c r="B329" s="11" t="n"/>
+      <c r="C329" s="11" t="n"/>
+      <c r="D329" s="11" t="n"/>
+      <c r="E329" s="11" t="n"/>
+      <c r="F329" s="42" t="n"/>
       <c r="G329" s="53" t="n"/>
     </row>
-    <row r="330" ht="19.8" customHeight="1">
-      <c r="A330" s="8" t="inlineStr">
-        <is>
-          <t>LOCAL  17 - Bano   (PA)   -   altura 3.00 m</t>
-        </is>
-      </c>
-      <c r="B330" s="11" t="n"/>
-      <c r="C330" s="11" t="n"/>
-      <c r="D330" s="11" t="n"/>
-      <c r="E330" s="11" t="n"/>
-      <c r="F330" s="42" t="n"/>
+    <row r="330" ht="32" customHeight="1">
+      <c r="A330" s="2" t="inlineStr">
+        <is>
+          <t>Nro</t>
+        </is>
+      </c>
+      <c r="B330" s="2" t="inlineStr">
+        <is>
+          <t>DESCRIPCION</t>
+        </is>
+      </c>
+      <c r="C330" s="2" t="inlineStr">
+        <is>
+          <t>DIMENSIONES (m)</t>
+        </is>
+      </c>
+      <c r="D330" s="2" t="inlineStr">
+        <is>
+          <t>AREA (m2)</t>
+        </is>
+      </c>
+      <c r="E330" s="2" t="inlineStr">
+        <is>
+          <t>FACTOR</t>
+        </is>
+      </c>
+      <c r="F330" s="2" t="inlineStr">
+        <is>
+          <t>PERDIDA CALOR (Kcal/h)</t>
+        </is>
+      </c>
       <c r="G330" s="53" t="n"/>
     </row>
-    <row r="331" ht="32" customHeight="1">
-      <c r="A331" s="2" t="inlineStr">
-        <is>
-          <t>Nro</t>
-        </is>
-      </c>
-      <c r="B331" s="2" t="inlineStr">
-        <is>
-          <t>DESCRIPCION</t>
-        </is>
-      </c>
-      <c r="C331" s="2" t="inlineStr">
-        <is>
-          <t>DIMENSIONES (m)</t>
-        </is>
-      </c>
-      <c r="D331" s="2" t="inlineStr">
-        <is>
-          <t>AREA (m2)</t>
-        </is>
-      </c>
-      <c r="E331" s="2" t="inlineStr">
-        <is>
-          <t>FACTOR</t>
-        </is>
-      </c>
-      <c r="F331" s="2" t="inlineStr">
-        <is>
-          <t>PERDIDA CALOR (Kcal/h)</t>
-        </is>
-      </c>
+    <row r="331" ht="19.8" customHeight="1">
+      <c r="A331" s="36" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="B331" s="78" t="inlineStr">
+        <is>
+          <t>VENTANA</t>
+        </is>
+      </c>
+      <c r="C331" s="43" t="n"/>
+      <c r="D331" s="58" t="n"/>
+      <c r="E331" s="58" t="n"/>
+      <c r="F331" s="61" t="n"/>
       <c r="G331" s="53" t="n"/>
     </row>
     <row r="332" ht="19.8" customHeight="1">
-      <c r="A332" s="36" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="B332" s="78" t="inlineStr">
-        <is>
-          <t>VENTANA</t>
-        </is>
-      </c>
-      <c r="C332" s="43" t="n"/>
-      <c r="D332" s="58" t="n"/>
-      <c r="E332" s="58" t="n"/>
-      <c r="F332" s="61" t="n"/>
+      <c r="A332" s="90" t="n"/>
+      <c r="B332" s="91" t="inlineStr">
+        <is>
+          <t>VA03</t>
+        </is>
+      </c>
+      <c r="C332" s="18" t="inlineStr">
+        <is>
+          <t>0.75 x 2.52</t>
+        </is>
+      </c>
+      <c r="D332" s="19" t="n">
+        <v>1.89</v>
+      </c>
+      <c r="E332" s="59" t="n">
+        <v>60</v>
+      </c>
+      <c r="F332" s="80" t="n">
+        <v>113.4</v>
+      </c>
       <c r="G332" s="53" t="n"/>
     </row>
     <row r="333" ht="19.8" customHeight="1">
-      <c r="A333" s="90" t="n"/>
-      <c r="B333" s="91" t="inlineStr">
-        <is>
-          <t>VA03</t>
-        </is>
-      </c>
-      <c r="C333" s="18" t="inlineStr">
-        <is>
-          <t>0.75 x 2.52</t>
-        </is>
-      </c>
-      <c r="D333" s="19" t="n">
-        <v>1.89</v>
-      </c>
-      <c r="E333" s="59" t="n">
-        <v>60</v>
-      </c>
-      <c r="F333" s="80" t="n">
-        <v>113.4</v>
-      </c>
+      <c r="A333" s="36" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="B333" s="78" t="inlineStr">
+        <is>
+          <t>PAREDES EXTERIORES</t>
+        </is>
+      </c>
+      <c r="C333" s="47" t="n"/>
+      <c r="D333" s="18" t="n"/>
+      <c r="E333" s="18" t="n"/>
+      <c r="F333" s="20" t="n"/>
       <c r="G333" s="53" t="n"/>
     </row>
     <row r="334" ht="19.8" customHeight="1">
-      <c r="A334" s="36" t="inlineStr">
-        <is>
-          <t>2</t>
-        </is>
-      </c>
-      <c r="B334" s="78" t="inlineStr">
-        <is>
-          <t>PAREDES EXTERIORES</t>
-        </is>
-      </c>
-      <c r="C334" s="47" t="n"/>
-      <c r="D334" s="18" t="n"/>
-      <c r="E334" s="18" t="n"/>
-      <c r="F334" s="20" t="n"/>
+      <c r="A334" s="43" t="n"/>
+      <c r="B334" s="79" t="inlineStr">
+        <is>
+          <t>AISLADAS (NE)</t>
+        </is>
+      </c>
+      <c r="C334" s="18" t="inlineStr">
+        <is>
+          <t>2.20 x 3.00</t>
+        </is>
+      </c>
+      <c r="D334" s="19" t="n">
+        <v>6.6</v>
+      </c>
+      <c r="E334" s="59" t="n">
+        <v>20</v>
+      </c>
+      <c r="F334" s="80" t="n">
+        <v>132</v>
+      </c>
       <c r="G334" s="53" t="n"/>
     </row>
     <row r="335" ht="19.8" customHeight="1">
-      <c r="A335" s="43" t="n"/>
-      <c r="B335" s="79" t="inlineStr">
-        <is>
-          <t>AISLADAS (NE)</t>
+      <c r="A335" s="47" t="n"/>
+      <c r="B335" s="81" t="inlineStr">
+        <is>
+          <t>AISLADAS</t>
         </is>
       </c>
       <c r="C335" s="18" t="inlineStr">
         <is>
-          <t>2.20 x 3.00</t>
+          <t>1.60 x 3.00</t>
         </is>
       </c>
       <c r="D335" s="19" t="n">
-        <v>6.6</v>
+        <v>4.8</v>
       </c>
       <c r="E335" s="59" t="n">
         <v>20</v>
       </c>
       <c r="F335" s="80" t="n">
-        <v>132</v>
+        <v>96</v>
       </c>
       <c r="G335" s="53" t="n"/>
     </row>
@@ -26026,366 +26026,358 @@
       <c r="A336" s="47" t="n"/>
       <c r="B336" s="81" t="inlineStr">
         <is>
-          <t>AISLADAS</t>
+          <t>INTERIORES (SO)</t>
         </is>
       </c>
       <c r="C336" s="18" t="inlineStr">
         <is>
+          <t>2.20 x 3.00</t>
+        </is>
+      </c>
+      <c r="D336" s="19" t="n">
+        <v>6.6</v>
+      </c>
+      <c r="E336" s="59" t="n">
+        <v>25</v>
+      </c>
+      <c r="F336" s="80" t="n">
+        <v>165</v>
+      </c>
+      <c r="G336" s="53" t="n"/>
+    </row>
+    <row r="337" ht="19.8" customHeight="1">
+      <c r="A337" s="50" t="n"/>
+      <c r="B337" s="82" t="inlineStr">
+        <is>
+          <t>INTERIORES</t>
+        </is>
+      </c>
+      <c r="C337" s="18" t="inlineStr">
+        <is>
           <t>1.60 x 3.00</t>
         </is>
       </c>
-      <c r="D336" s="19" t="n">
+      <c r="D337" s="19" t="n">
         <v>4.8</v>
-      </c>
-      <c r="E336" s="59" t="n">
-        <v>20</v>
-      </c>
-      <c r="F336" s="80" t="n">
-        <v>96</v>
-      </c>
-      <c r="G336" s="53" t="n"/>
-    </row>
-    <row r="337" ht="19.8" customHeight="1">
-      <c r="A337" s="47" t="n"/>
-      <c r="B337" s="81" t="inlineStr">
-        <is>
-          <t>INTERIORES (SO)</t>
-        </is>
-      </c>
-      <c r="C337" s="18" t="inlineStr">
-        <is>
-          <t>2.20 x 3.00</t>
-        </is>
-      </c>
-      <c r="D337" s="19" t="n">
-        <v>6.6</v>
       </c>
       <c r="E337" s="59" t="n">
         <v>25</v>
       </c>
       <c r="F337" s="80" t="n">
-        <v>165</v>
+        <v>120</v>
       </c>
       <c r="G337" s="53" t="n"/>
     </row>
     <row r="338" ht="19.8" customHeight="1">
-      <c r="A338" s="50" t="n"/>
-      <c r="B338" s="82" t="inlineStr">
-        <is>
-          <t>INTERIORES</t>
-        </is>
-      </c>
-      <c r="C338" s="18" t="inlineStr">
-        <is>
-          <t>1.60 x 3.00</t>
-        </is>
-      </c>
-      <c r="D338" s="19" t="n">
-        <v>4.8</v>
-      </c>
-      <c r="E338" s="59" t="n">
-        <v>25</v>
-      </c>
-      <c r="F338" s="80" t="n">
-        <v>120</v>
-      </c>
+      <c r="A338" s="36" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="B338" s="78" t="inlineStr">
+        <is>
+          <t>TECHOS O CIELORRASOS</t>
+        </is>
+      </c>
+      <c r="C338" s="47" t="n"/>
+      <c r="D338" s="18" t="n"/>
+      <c r="E338" s="18" t="n"/>
+      <c r="F338" s="20" t="n"/>
       <c r="G338" s="53" t="n"/>
     </row>
     <row r="339" ht="19.8" customHeight="1">
-      <c r="A339" s="36" t="inlineStr">
-        <is>
-          <t>3</t>
-        </is>
-      </c>
-      <c r="B339" s="78" t="inlineStr">
-        <is>
-          <t>TECHOS O CIELORRASOS</t>
-        </is>
-      </c>
-      <c r="C339" s="47" t="n"/>
-      <c r="D339" s="18" t="n"/>
-      <c r="E339" s="18" t="n"/>
-      <c r="F339" s="20" t="n"/>
+      <c r="A339" s="43" t="n"/>
+      <c r="B339" s="79" t="inlineStr">
+        <is>
+          <t>TECHO NO AISLADO</t>
+        </is>
+      </c>
+      <c r="C339" s="18" t="n"/>
+      <c r="D339" s="19" t="n"/>
+      <c r="E339" s="59" t="n">
+        <v>30</v>
+      </c>
+      <c r="F339" s="80" t="n"/>
       <c r="G339" s="53" t="n"/>
     </row>
     <row r="340" ht="19.8" customHeight="1">
-      <c r="A340" s="43" t="n"/>
-      <c r="B340" s="79" t="inlineStr">
-        <is>
-          <t>TECHO NO AISLADO</t>
-        </is>
-      </c>
-      <c r="C340" s="18" t="n"/>
-      <c r="D340" s="19" t="n"/>
+      <c r="A340" s="47" t="n"/>
+      <c r="B340" s="81" t="inlineStr">
+        <is>
+          <t>TECHO AISLADO</t>
+        </is>
+      </c>
+      <c r="C340" s="18" t="inlineStr">
+        <is>
+          <t>por croquis</t>
+        </is>
+      </c>
+      <c r="D340" s="19" t="n">
+        <v>3.52</v>
+      </c>
       <c r="E340" s="59" t="n">
-        <v>30</v>
-      </c>
-      <c r="F340" s="80" t="n"/>
+        <v>20</v>
+      </c>
+      <c r="F340" s="80" t="n">
+        <v>70.40000000000001</v>
+      </c>
       <c r="G340" s="53" t="n"/>
     </row>
     <row r="341" ht="19.8" customHeight="1">
-      <c r="A341" s="47" t="n"/>
-      <c r="B341" s="81" t="inlineStr">
-        <is>
-          <t>TECHO AISLADO</t>
-        </is>
-      </c>
-      <c r="C341" s="18" t="inlineStr">
+      <c r="A341" s="50" t="n"/>
+      <c r="B341" s="82" t="inlineStr">
+        <is>
+          <t>TECHO ENTREPISO</t>
+        </is>
+      </c>
+      <c r="C341" s="18" t="n"/>
+      <c r="D341" s="19" t="n"/>
+      <c r="E341" s="59" t="n">
+        <v>15</v>
+      </c>
+      <c r="F341" s="80" t="n"/>
+      <c r="G341" s="53" t="n"/>
+    </row>
+    <row r="342" ht="19.8" customHeight="1">
+      <c r="A342" s="36" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="B342" s="78" t="inlineStr">
+        <is>
+          <t>PISO</t>
+        </is>
+      </c>
+      <c r="C342" s="47" t="n"/>
+      <c r="D342" s="18" t="n"/>
+      <c r="E342" s="18" t="n"/>
+      <c r="F342" s="20" t="n"/>
+      <c r="G342" s="53" t="n"/>
+    </row>
+    <row r="343" ht="19.8" customHeight="1">
+      <c r="A343" s="43" t="n"/>
+      <c r="B343" s="79" t="inlineStr">
+        <is>
+          <t>SOBRE TIERRA</t>
+        </is>
+      </c>
+      <c r="C343" s="18" t="n"/>
+      <c r="D343" s="19" t="n"/>
+      <c r="E343" s="59" t="n">
+        <v>10</v>
+      </c>
+      <c r="F343" s="80" t="n"/>
+      <c r="G343" s="53" t="n"/>
+    </row>
+    <row r="344" ht="19.8" customHeight="1">
+      <c r="A344" s="50" t="n"/>
+      <c r="B344" s="82" t="inlineStr">
+        <is>
+          <t>SOBRE LOCAL OCUPADO</t>
+        </is>
+      </c>
+      <c r="C344" s="18" t="inlineStr">
         <is>
           <t>por croquis</t>
         </is>
       </c>
-      <c r="D341" s="19" t="n">
+      <c r="D344" s="24" t="n">
         <v>3.52</v>
       </c>
-      <c r="E341" s="59" t="n">
-        <v>20</v>
-      </c>
-      <c r="F341" s="80" t="n">
-        <v>70.40000000000001</v>
-      </c>
-      <c r="G341" s="53" t="n"/>
-    </row>
-    <row r="342" ht="19.8" customHeight="1">
-      <c r="A342" s="50" t="n"/>
-      <c r="B342" s="82" t="inlineStr">
-        <is>
-          <t>TECHO ENTREPISO</t>
-        </is>
-      </c>
-      <c r="C342" s="18" t="n"/>
-      <c r="D342" s="19" t="n"/>
-      <c r="E342" s="59" t="n">
+      <c r="E344" s="59" t="n">
         <v>15</v>
       </c>
-      <c r="F342" s="80" t="n"/>
-      <c r="G342" s="53" t="n"/>
-    </row>
-    <row r="343" ht="19.8" customHeight="1">
-      <c r="A343" s="36" t="inlineStr">
-        <is>
-          <t>4</t>
-        </is>
-      </c>
-      <c r="B343" s="78" t="inlineStr">
-        <is>
-          <t>PISO</t>
-        </is>
-      </c>
-      <c r="C343" s="47" t="n"/>
-      <c r="D343" s="18" t="n"/>
-      <c r="E343" s="18" t="n"/>
-      <c r="F343" s="20" t="n"/>
-      <c r="G343" s="53" t="n"/>
-    </row>
-    <row r="344" ht="19.8" customHeight="1">
-      <c r="A344" s="43" t="n"/>
-      <c r="B344" s="79" t="inlineStr">
-        <is>
-          <t>SOBRE TIERRA</t>
-        </is>
-      </c>
-      <c r="C344" s="18" t="n"/>
-      <c r="D344" s="19" t="n"/>
-      <c r="E344" s="59" t="n">
-        <v>10</v>
-      </c>
-      <c r="F344" s="80" t="n"/>
+      <c r="F344" s="80" t="n">
+        <v>52.8</v>
+      </c>
       <c r="G344" s="53" t="n"/>
     </row>
     <row r="345" ht="19.8" customHeight="1">
-      <c r="A345" s="50" t="n"/>
-      <c r="B345" s="82" t="inlineStr">
-        <is>
-          <t>SOBRE LOCAL OCUPADO</t>
-        </is>
-      </c>
-      <c r="C345" s="18" t="inlineStr">
-        <is>
-          <t>por croquis</t>
-        </is>
-      </c>
-      <c r="D345" s="24" t="n">
-        <v>3.52</v>
-      </c>
-      <c r="E345" s="59" t="n">
-        <v>15</v>
-      </c>
-      <c r="F345" s="80" t="n">
-        <v>52.8</v>
-      </c>
+      <c r="A345" s="36" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="B345" s="78" t="inlineStr">
+        <is>
+          <t>INFILTRACION</t>
+        </is>
+      </c>
+      <c r="C345" s="83" t="n"/>
+      <c r="D345" s="36" t="inlineStr">
+        <is>
+          <t>VOLUMEN (m3)</t>
+        </is>
+      </c>
+      <c r="E345" s="47" t="n"/>
+      <c r="F345" s="20" t="n"/>
       <c r="G345" s="53" t="n"/>
     </row>
     <row r="346" ht="19.8" customHeight="1">
-      <c r="A346" s="36" t="inlineStr">
-        <is>
-          <t>5</t>
-        </is>
-      </c>
-      <c r="B346" s="78" t="inlineStr">
-        <is>
-          <t>INFILTRACION</t>
-        </is>
-      </c>
-      <c r="C346" s="83" t="n"/>
-      <c r="D346" s="36" t="inlineStr">
-        <is>
-          <t>VOLUMEN (m3)</t>
-        </is>
-      </c>
-      <c r="E346" s="47" t="n"/>
-      <c r="F346" s="20" t="n"/>
+      <c r="A346" s="43" t="n"/>
+      <c r="B346" s="79" t="inlineStr">
+        <is>
+          <t>UNA PARED EXTERIOR</t>
+        </is>
+      </c>
+      <c r="C346" s="18" t="n"/>
+      <c r="D346" s="22" t="n"/>
+      <c r="E346" s="59" t="n">
+        <v>6</v>
+      </c>
+      <c r="F346" s="80" t="n"/>
       <c r="G346" s="53" t="n"/>
     </row>
     <row r="347" ht="19.8" customHeight="1">
-      <c r="A347" s="43" t="n"/>
-      <c r="B347" s="79" t="inlineStr">
-        <is>
-          <t>UNA PARED EXTERIOR</t>
-        </is>
-      </c>
-      <c r="C347" s="18" t="n"/>
-      <c r="D347" s="22" t="n"/>
+      <c r="A347" s="47" t="n"/>
+      <c r="B347" s="81" t="inlineStr">
+        <is>
+          <t>DOS PAREDES EXTERIORES</t>
+        </is>
+      </c>
+      <c r="C347" s="18" t="inlineStr">
+        <is>
+          <t>3.52 m2 x 3.00</t>
+        </is>
+      </c>
+      <c r="D347" s="19" t="n">
+        <v>10.56</v>
+      </c>
       <c r="E347" s="59" t="n">
-        <v>6</v>
-      </c>
-      <c r="F347" s="80" t="n"/>
+        <v>9</v>
+      </c>
+      <c r="F347" s="80" t="n">
+        <v>95</v>
+      </c>
       <c r="G347" s="53" t="n"/>
     </row>
     <row r="348" ht="19.8" customHeight="1">
-      <c r="A348" s="47" t="n"/>
-      <c r="B348" s="81" t="inlineStr">
-        <is>
-          <t>DOS PAREDES EXTERIORES</t>
-        </is>
-      </c>
-      <c r="C348" s="18" t="inlineStr">
-        <is>
-          <t>3.52 m2 x 3.00</t>
-        </is>
-      </c>
-      <c r="D348" s="19" t="n">
-        <v>10.56</v>
-      </c>
+      <c r="A348" s="50" t="n"/>
+      <c r="B348" s="82" t="inlineStr">
+        <is>
+          <t>TRES O MAS PAREDES EXTERIORES</t>
+        </is>
+      </c>
+      <c r="C348" s="18" t="n"/>
+      <c r="D348" s="19" t="n"/>
       <c r="E348" s="59" t="n">
-        <v>9</v>
-      </c>
-      <c r="F348" s="80" t="n">
-        <v>95</v>
-      </c>
+        <v>12</v>
+      </c>
+      <c r="F348" s="84" t="n"/>
       <c r="G348" s="53" t="n"/>
     </row>
     <row r="349" ht="19.8" customHeight="1">
-      <c r="A349" s="50" t="n"/>
-      <c r="B349" s="82" t="inlineStr">
-        <is>
-          <t>TRES O MAS PAREDES EXTERIORES</t>
-        </is>
-      </c>
-      <c r="C349" s="18" t="n"/>
-      <c r="D349" s="19" t="n"/>
-      <c r="E349" s="59" t="n">
-        <v>12</v>
-      </c>
-      <c r="F349" s="84" t="n"/>
+      <c r="A349" s="36" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="B349" s="78" t="inlineStr">
+        <is>
+          <t>SUBTOTAL</t>
+        </is>
+      </c>
+      <c r="C349" s="47" t="n"/>
+      <c r="D349" s="18" t="n"/>
+      <c r="E349" s="20" t="n"/>
+      <c r="F349" s="85" t="n">
+        <v>844.6</v>
+      </c>
       <c r="G349" s="53" t="n"/>
     </row>
     <row r="350" ht="19.8" customHeight="1">
       <c r="A350" s="36" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B350" s="78" t="inlineStr">
         <is>
-          <t>SUBTOTAL</t>
-        </is>
-      </c>
-      <c r="C350" s="47" t="n"/>
-      <c r="D350" s="18" t="n"/>
-      <c r="E350" s="20" t="n"/>
+          <t>PERDIDA TOTAL</t>
+        </is>
+      </c>
+      <c r="C350" s="47" t="inlineStr">
+        <is>
+          <t>844.60  X  1.07 (FI)  X  1 (FO)  X  1 (FZ)</t>
+        </is>
+      </c>
+      <c r="D350" s="12" t="n"/>
+      <c r="E350" s="14" t="n"/>
       <c r="F350" s="85" t="n">
-        <v>844.6</v>
+        <v>903.7</v>
       </c>
       <c r="G350" s="53" t="n"/>
     </row>
     <row r="351" ht="19.8" customHeight="1">
-      <c r="A351" s="36" t="inlineStr">
-        <is>
-          <t>7</t>
-        </is>
-      </c>
-      <c r="B351" s="78" t="inlineStr">
-        <is>
-          <t>PERDIDA TOTAL</t>
-        </is>
-      </c>
-      <c r="C351" s="47" t="inlineStr">
-        <is>
-          <t>844.60  X  1.07 (FI)  X  1 (FO)  X  1 (FZ)</t>
-        </is>
-      </c>
+      <c r="A351" s="43" t="n"/>
+      <c r="B351" s="86" t="inlineStr">
+        <is>
+          <t>Carga de locales sin emisor</t>
+        </is>
+      </c>
+      <c r="C351" s="18" t="n"/>
       <c r="D351" s="12" t="n"/>
-      <c r="E351" s="14" t="n"/>
-      <c r="F351" s="85" t="n">
+      <c r="E351" s="39" t="n"/>
+      <c r="F351" s="87" t="n"/>
+      <c r="G351" s="53" t="n"/>
+    </row>
+    <row r="352" ht="19.8" customHeight="1">
+      <c r="A352" s="83" t="n"/>
+      <c r="B352" s="78" t="inlineStr">
+        <is>
+          <t>CARGA TOTAL A CUBRIR</t>
+        </is>
+      </c>
+      <c r="C352" s="47" t="n"/>
+      <c r="D352" s="12" t="n"/>
+      <c r="E352" s="14" t="n"/>
+      <c r="F352" s="85" t="n">
         <v>903.7</v>
       </c>
-      <c r="G351" s="53" t="n"/>
-    </row>
-    <row r="352" ht="19.8" customHeight="1">
-      <c r="A352" s="43" t="n"/>
-      <c r="B352" s="86" t="inlineStr">
-        <is>
-          <t>Carga de locales sin emisor</t>
-        </is>
-      </c>
-      <c r="C352" s="18" t="n"/>
-      <c r="D352" s="12" t="n"/>
-      <c r="E352" s="39" t="n"/>
-      <c r="F352" s="87" t="n"/>
       <c r="G352" s="53" t="n"/>
     </row>
     <row r="353" ht="19.8" customHeight="1">
-      <c r="A353" s="83" t="n"/>
-      <c r="B353" s="78" t="inlineStr">
-        <is>
-          <t>CARGA TOTAL A CUBRIR</t>
-        </is>
-      </c>
-      <c r="C353" s="47" t="n"/>
+      <c r="A353" s="47" t="n"/>
+      <c r="B353" s="88" t="inlineStr">
+        <is>
+          <t>Salto termico:  dt = (te+ts)/2 - ti</t>
+        </is>
+      </c>
+      <c r="C353" s="18" t="inlineStr">
+        <is>
+          <t>86 - 20 = 66 C</t>
+        </is>
+      </c>
       <c r="D353" s="12" t="n"/>
-      <c r="E353" s="14" t="n"/>
-      <c r="F353" s="85" t="n">
-        <v>903.7</v>
-      </c>
+      <c r="E353" s="39" t="n"/>
+      <c r="F353" s="61" t="n"/>
       <c r="G353" s="53" t="n"/>
     </row>
     <row r="354" ht="19.8" customHeight="1">
       <c r="A354" s="47" t="n"/>
-      <c r="B354" s="88" t="inlineStr">
-        <is>
-          <t>Salto termico:  dt = (te+ts)/2 - ti</t>
-        </is>
-      </c>
-      <c r="C354" s="18" t="inlineStr">
-        <is>
-          <t>86 - 20 = 66 C</t>
-        </is>
+      <c r="B354" s="60" t="inlineStr">
+        <is>
+          <t>Kcal/h del toallero Scala/Domino 80</t>
+        </is>
+      </c>
+      <c r="C354" s="59" t="n">
+        <v>708</v>
       </c>
       <c r="D354" s="12" t="n"/>
       <c r="E354" s="39" t="n"/>
-      <c r="F354" s="61" t="n"/>
+      <c r="F354" s="20" t="n"/>
       <c r="G354" s="53" t="n"/>
     </row>
     <row r="355" ht="19.8" customHeight="1">
       <c r="A355" s="47" t="n"/>
       <c r="B355" s="60" t="inlineStr">
         <is>
-          <t>Kcal/h del toallero Scala/Domino 80</t>
+          <t>Kcal/h del toallero Scala/Domino 150</t>
         </is>
       </c>
       <c r="C355" s="59" t="n">
-        <v>708</v>
+        <v>1315</v>
       </c>
       <c r="D355" s="12" t="n"/>
       <c r="E355" s="39" t="n"/>
@@ -26396,11 +26388,11 @@
       <c r="A356" s="47" t="n"/>
       <c r="B356" s="60" t="inlineStr">
         <is>
-          <t>Kcal/h del toallero Scala/Domino 150</t>
+          <t>Toalleros necesarios</t>
         </is>
       </c>
       <c r="C356" s="59" t="n">
-        <v>1315</v>
+        <v>1</v>
       </c>
       <c r="D356" s="12" t="n"/>
       <c r="E356" s="39" t="n"/>
@@ -26408,51 +26400,37 @@
       <c r="G356" s="53" t="n"/>
     </row>
     <row r="357" ht="19.8" customHeight="1">
-      <c r="A357" s="47" t="n"/>
-      <c r="B357" s="60" t="inlineStr">
-        <is>
-          <t>Toalleros necesarios</t>
-        </is>
-      </c>
-      <c r="C357" s="59" t="n">
-        <v>1</v>
-      </c>
-      <c r="D357" s="12" t="n"/>
-      <c r="E357" s="39" t="n"/>
-      <c r="F357" s="20" t="n"/>
+      <c r="A357" s="50" t="n"/>
+      <c r="B357" s="72" t="inlineStr">
+        <is>
+          <t>Toallero adoptado</t>
+        </is>
+      </c>
+      <c r="C357" s="30" t="inlineStr">
+        <is>
+          <t>Peisa Scala / Domino 150  (500 x 1500 mm)</t>
+        </is>
+      </c>
+      <c r="D357" s="11" t="n"/>
+      <c r="E357" s="92" t="n"/>
+      <c r="F357" s="31" t="n"/>
       <c r="G357" s="53" t="n"/>
-    </row>
-    <row r="358" ht="19.8" customHeight="1">
-      <c r="A358" s="50" t="n"/>
-      <c r="B358" s="72" t="inlineStr">
-        <is>
-          <t>Toallero adoptado</t>
-        </is>
-      </c>
-      <c r="C358" s="30" t="inlineStr">
-        <is>
-          <t>Peisa Scala / Domino 150  (500 x 1500 mm)</t>
-        </is>
-      </c>
-      <c r="D358" s="11" t="n"/>
-      <c r="E358" s="92" t="n"/>
-      <c r="F358" s="31" t="n"/>
-      <c r="G358" s="53" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="101">
+    <mergeCell ref="C321:E321"/>
     <mergeCell ref="C202:E202"/>
     <mergeCell ref="C31:E31"/>
-    <mergeCell ref="C329:E329"/>
-    <mergeCell ref="A301:F301"/>
     <mergeCell ref="C297:E297"/>
     <mergeCell ref="C60:E60"/>
     <mergeCell ref="C123:E123"/>
     <mergeCell ref="C268:E268"/>
     <mergeCell ref="C299:E299"/>
+    <mergeCell ref="C292:E292"/>
     <mergeCell ref="C57:E57"/>
     <mergeCell ref="C355:E355"/>
     <mergeCell ref="C293:E293"/>
+    <mergeCell ref="A329:F329"/>
     <mergeCell ref="C204:E204"/>
     <mergeCell ref="C357:E357"/>
     <mergeCell ref="C325:E325"/>
@@ -26493,12 +26471,11 @@
     <mergeCell ref="C324:E324"/>
     <mergeCell ref="C63:E63"/>
     <mergeCell ref="C121:E121"/>
-    <mergeCell ref="A330:F330"/>
     <mergeCell ref="C117:E117"/>
     <mergeCell ref="C173:E173"/>
     <mergeCell ref="C236:E236"/>
     <mergeCell ref="A210:F210"/>
-    <mergeCell ref="C300:E300"/>
+    <mergeCell ref="C350:E350"/>
     <mergeCell ref="C207:E207"/>
     <mergeCell ref="C328:E328"/>
     <mergeCell ref="C122:E122"/>
@@ -26513,6 +26490,7 @@
     <mergeCell ref="C30:E30"/>
     <mergeCell ref="C235:E235"/>
     <mergeCell ref="C62:E62"/>
+    <mergeCell ref="A300:F300"/>
     <mergeCell ref="C234:E234"/>
     <mergeCell ref="A1:F1"/>
     <mergeCell ref="C172:E172"/>
@@ -26531,7 +26509,6 @@
     <mergeCell ref="C119:E119"/>
     <mergeCell ref="A91:F91"/>
     <mergeCell ref="C174:E174"/>
-    <mergeCell ref="C358:E358"/>
     <mergeCell ref="C327:E327"/>
     <mergeCell ref="C237:E237"/>
     <mergeCell ref="C351:E351"/>

</xml_diff>

<commit_message>
Living: paredes de 4,06 con orientacion (NE cocina, SO escalera)
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01NNMcFTBbEuLfDho1wCZzu7
</commit_message>
<xml_diff>
--- a/planillas/planillas_estructura (para AutoCAD).xlsx
+++ b/planillas/planillas_estructura (para AutoCAD).xlsx
@@ -20496,7 +20496,7 @@
       <c r="A42" s="47" t="n"/>
       <c r="B42" s="81" t="inlineStr">
         <is>
-          <t>INTERIORES (cocina)</t>
+          <t>INTERIORES (NE, cocina)</t>
         </is>
       </c>
       <c r="C42" s="18" t="inlineStr">
@@ -20542,7 +20542,7 @@
       <c r="A44" s="50" t="n"/>
       <c r="B44" s="82" t="inlineStr">
         <is>
-          <t>INTERIORES (escalera)</t>
+          <t>INTERIORES (SO, escalera)</t>
         </is>
       </c>
       <c r="C44" s="18" t="inlineStr">

</xml_diff>

<commit_message>
Escalera: la 1,73 aislada es SO y la interior NE
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01NNMcFTBbEuLfDho1wCZzu7
</commit_message>
<xml_diff>
--- a/planillas/planillas_estructura (para AutoCAD).xlsx
+++ b/planillas/planillas_estructura (para AutoCAD).xlsx
@@ -22145,7 +22145,7 @@
       <c r="A129" s="43" t="n"/>
       <c r="B129" s="79" t="inlineStr">
         <is>
-          <t>AISLADAS (NE)</t>
+          <t>AISLADAS</t>
         </is>
       </c>
       <c r="C129" s="18" t="inlineStr">
@@ -22168,7 +22168,7 @@
       <c r="A130" s="47" t="n"/>
       <c r="B130" s="81" t="inlineStr">
         <is>
-          <t>AISLADAS</t>
+          <t>AISLADAS (SO)</t>
         </is>
       </c>
       <c r="C130" s="18" t="inlineStr">
@@ -22191,7 +22191,7 @@
       <c r="A131" s="47" t="n"/>
       <c r="B131" s="81" t="inlineStr">
         <is>
-          <t>INTERIORES (SO)</t>
+          <t>INTERIORES</t>
         </is>
       </c>
       <c r="C131" s="18" t="inlineStr">
@@ -22214,7 +22214,7 @@
       <c r="A132" s="50" t="n"/>
       <c r="B132" s="82" t="inlineStr">
         <is>
-          <t>INTERIORES</t>
+          <t>INTERIORES (NE)</t>
         </is>
       </c>
       <c r="C132" s="18" t="inlineStr">

</xml_diff>

<commit_message>
Balance termico: los rotulos de las paredes no llevan aberturas
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01NNMcFTBbEuLfDho1wCZzu7
</commit_message>
<xml_diff>
--- a/planillas/planillas_estructura (para AutoCAD).xlsx
+++ b/planillas/planillas_estructura (para AutoCAD).xlsx
@@ -20519,7 +20519,7 @@
       <c r="A43" s="47" t="n"/>
       <c r="B43" s="81" t="inlineStr">
         <is>
-          <t>INTERIORES (NO, galeria, con la PV01)</t>
+          <t>INTERIORES (NO, galeria)</t>
         </is>
       </c>
       <c r="C43" s="18" t="inlineStr">
@@ -21556,7 +21556,7 @@
       <c r="A98" s="47" t="n"/>
       <c r="B98" s="81" t="inlineStr">
         <is>
-          <t>INTERIORES (resto del lado largo)</t>
+          <t>INTERIORES</t>
         </is>
       </c>
       <c r="C98" s="18" t="inlineStr">

</xml_diff>

<commit_message>
Version para AutoCAD: se conservan los esquemas de vigas, losas y vigas de fundacion
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01NNMcFTBbEuLfDho1wCZzu7
</commit_message>
<xml_diff>
--- a/planillas/planillas_estructura (para AutoCAD).xlsx
+++ b/planillas/planillas_estructura (para AutoCAD).xlsx
@@ -983,6 +983,1901 @@
 </styleSheet>
 </file>
 
+<file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
+<wsDr xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+  <oneCellAnchor>
+    <from>
+      <col>0</col>
+      <colOff>0</colOff>
+      <row>0</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="2743200" cy="3276600"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="1" name="Image 1" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId1"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+</wsDr>
+</file>
+
+<file path=xl/drawings/drawing2.xml><?xml version="1.0" encoding="utf-8"?>
+<wsDr xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+  <oneCellAnchor>
+    <from>
+      <col>4</col>
+      <colOff>0</colOff>
+      <row>3</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="2095500" cy="571500"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="1" name="Image 1" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId1"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>4</col>
+      <colOff>0</colOff>
+      <row>4</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="2095500" cy="571500"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="2" name="Image 2" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId2"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>4</col>
+      <colOff>0</colOff>
+      <row>5</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="2095500" cy="571500"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="3" name="Image 3" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId3"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>4</col>
+      <colOff>0</colOff>
+      <row>6</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="2095500" cy="571500"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="4" name="Image 4" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId4"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>4</col>
+      <colOff>0</colOff>
+      <row>7</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="2095500" cy="571500"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="5" name="Image 5" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId5"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>4</col>
+      <colOff>0</colOff>
+      <row>8</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="2095500" cy="571500"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="6" name="Image 6" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId6"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>4</col>
+      <colOff>0</colOff>
+      <row>9</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="2095500" cy="571500"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="7" name="Image 7" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId7"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>4</col>
+      <colOff>0</colOff>
+      <row>10</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="2095500" cy="571500"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="8" name="Image 8" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId8"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>4</col>
+      <colOff>0</colOff>
+      <row>11</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="2095500" cy="571500"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="9" name="Image 9" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId9"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>4</col>
+      <colOff>0</colOff>
+      <row>12</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="2095500" cy="571500"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="10" name="Image 10" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId10"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>4</col>
+      <colOff>0</colOff>
+      <row>13</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="2095500" cy="571500"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="11" name="Image 11" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId11"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>4</col>
+      <colOff>0</colOff>
+      <row>14</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="2095500" cy="571500"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="12" name="Image 12" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId12"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>4</col>
+      <colOff>0</colOff>
+      <row>15</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="2095500" cy="571500"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="13" name="Image 13" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId13"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>4</col>
+      <colOff>0</colOff>
+      <row>16</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="2095500" cy="571500"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="14" name="Image 14" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId14"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>4</col>
+      <colOff>0</colOff>
+      <row>17</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="2095500" cy="571500"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="15" name="Image 15" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId15"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>4</col>
+      <colOff>0</colOff>
+      <row>18</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="2095500" cy="571500"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="16" name="Image 16" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId16"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>4</col>
+      <colOff>0</colOff>
+      <row>19</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="2095500" cy="571500"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="17" name="Image 17" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId17"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>4</col>
+      <colOff>0</colOff>
+      <row>20</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="2095500" cy="571500"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="18" name="Image 18" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId18"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>4</col>
+      <colOff>0</colOff>
+      <row>21</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="2095500" cy="571500"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="19" name="Image 19" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId19"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>4</col>
+      <colOff>0</colOff>
+      <row>22</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="2095500" cy="571500"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="20" name="Image 20" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId20"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>4</col>
+      <colOff>0</colOff>
+      <row>23</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="2095500" cy="571500"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="21" name="Image 21" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId21"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>4</col>
+      <colOff>0</colOff>
+      <row>24</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="2095500" cy="571500"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="22" name="Image 22" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId22"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>4</col>
+      <colOff>0</colOff>
+      <row>25</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="2095500" cy="571500"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="23" name="Image 23" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId23"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>4</col>
+      <colOff>0</colOff>
+      <row>26</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="2095500" cy="571500"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="24" name="Image 24" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId24"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>4</col>
+      <colOff>0</colOff>
+      <row>27</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="2095500" cy="571500"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="25" name="Image 25" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId25"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>4</col>
+      <colOff>0</colOff>
+      <row>28</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="2095500" cy="571500"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="26" name="Image 26" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId26"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>4</col>
+      <colOff>0</colOff>
+      <row>29</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="2095500" cy="571500"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="27" name="Image 27" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId27"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>4</col>
+      <colOff>0</colOff>
+      <row>30</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="2095500" cy="571500"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="28" name="Image 28" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId28"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>4</col>
+      <colOff>0</colOff>
+      <row>31</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="2095500" cy="571500"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="29" name="Image 29" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId29"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>4</col>
+      <colOff>0</colOff>
+      <row>32</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="2095500" cy="571500"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="30" name="Image 30" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId30"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>4</col>
+      <colOff>0</colOff>
+      <row>33</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="2095500" cy="571500"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="31" name="Image 31" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId31"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+</wsDr>
+</file>
+
+<file path=xl/drawings/drawing3.xml><?xml version="1.0" encoding="utf-8"?>
+<wsDr xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+  <oneCellAnchor>
+    <from>
+      <col>5</col>
+      <colOff>0</colOff>
+      <row>3</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="2095500" cy="571500"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="1" name="Image 1" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId1"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>5</col>
+      <colOff>0</colOff>
+      <row>4</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="2095500" cy="571500"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="2" name="Image 2" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId2"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>5</col>
+      <colOff>0</colOff>
+      <row>5</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="2095500" cy="571500"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="3" name="Image 3" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId3"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>5</col>
+      <colOff>0</colOff>
+      <row>6</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="2095500" cy="571500"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="4" name="Image 4" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId4"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>5</col>
+      <colOff>0</colOff>
+      <row>7</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="2095500" cy="571500"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="5" name="Image 5" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId5"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>5</col>
+      <colOff>0</colOff>
+      <row>8</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="2095500" cy="571500"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="6" name="Image 6" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId6"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>5</col>
+      <colOff>0</colOff>
+      <row>9</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="2095500" cy="571500"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="7" name="Image 7" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId7"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>5</col>
+      <colOff>0</colOff>
+      <row>10</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="2095500" cy="571500"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="8" name="Image 8" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId8"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>5</col>
+      <colOff>0</colOff>
+      <row>11</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="2095500" cy="571500"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="9" name="Image 9" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId9"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>5</col>
+      <colOff>0</colOff>
+      <row>12</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="2095500" cy="571500"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="10" name="Image 10" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId10"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>5</col>
+      <colOff>0</colOff>
+      <row>13</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="2095500" cy="571500"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="11" name="Image 11" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId11"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>5</col>
+      <colOff>0</colOff>
+      <row>14</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="2095500" cy="571500"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="12" name="Image 12" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId12"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+</wsDr>
+</file>
+
+<file path=xl/drawings/drawing4.xml><?xml version="1.0" encoding="utf-8"?>
+<wsDr xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+  <oneCellAnchor>
+    <from>
+      <col>4</col>
+      <colOff>0</colOff>
+      <row>3</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="2095500" cy="571500"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="1" name="Image 1" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId1"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>4</col>
+      <colOff>0</colOff>
+      <row>4</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="2095500" cy="571500"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="2" name="Image 2" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId2"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>4</col>
+      <colOff>0</colOff>
+      <row>5</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="2095500" cy="571500"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="3" name="Image 3" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId3"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>4</col>
+      <colOff>0</colOff>
+      <row>6</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="2095500" cy="571500"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="4" name="Image 4" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId4"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>4</col>
+      <colOff>0</colOff>
+      <row>7</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="2095500" cy="571500"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="5" name="Image 5" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId5"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>4</col>
+      <colOff>0</colOff>
+      <row>8</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="2095500" cy="571500"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="6" name="Image 6" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId6"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>4</col>
+      <colOff>0</colOff>
+      <row>9</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="2095500" cy="571500"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="7" name="Image 7" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId7"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>4</col>
+      <colOff>0</colOff>
+      <row>10</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="2095500" cy="571500"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="8" name="Image 8" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId8"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>4</col>
+      <colOff>0</colOff>
+      <row>11</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="2095500" cy="571500"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="9" name="Image 9" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId9"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>4</col>
+      <colOff>0</colOff>
+      <row>12</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="2095500" cy="571500"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="10" name="Image 10" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId10"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>4</col>
+      <colOff>0</colOff>
+      <row>13</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="2095500" cy="571500"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="11" name="Image 11" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId11"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>4</col>
+      <colOff>0</colOff>
+      <row>14</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="2095500" cy="571500"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="12" name="Image 12" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId12"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>4</col>
+      <colOff>0</colOff>
+      <row>15</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="2095500" cy="571500"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="13" name="Image 13" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId13"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>4</col>
+      <colOff>0</colOff>
+      <row>16</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="2095500" cy="571500"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="14" name="Image 14" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId14"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>4</col>
+      <colOff>0</colOff>
+      <row>17</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="2095500" cy="571500"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="15" name="Image 15" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId15"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>4</col>
+      <colOff>0</colOff>
+      <row>18</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="2095500" cy="571500"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="16" name="Image 16" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId16"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>4</col>
+      <colOff>0</colOff>
+      <row>19</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="2095500" cy="571500"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="17" name="Image 17" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId17"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>4</col>
+      <colOff>0</colOff>
+      <row>20</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="2095500" cy="571500"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="18" name="Image 18" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId18"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>4</col>
+      <colOff>0</colOff>
+      <row>21</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="2095500" cy="571500"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="19" name="Image 19" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId19"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>4</col>
+      <colOff>0</colOff>
+      <row>22</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="2095500" cy="571500"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="20" name="Image 20" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId20"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>4</col>
+      <colOff>0</colOff>
+      <row>23</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="2095500" cy="571500"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="21" name="Image 21" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId21"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>4</col>
+      <colOff>0</colOff>
+      <row>24</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="2095500" cy="571500"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="22" name="Image 22" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId22"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>4</col>
+      <colOff>0</colOff>
+      <row>25</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="2095500" cy="571500"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="23" name="Image 23" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId23"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>4</col>
+      <colOff>0</colOff>
+      <row>26</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="2095500" cy="571500"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="24" name="Image 24" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId24"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>4</col>
+      <colOff>0</colOff>
+      <row>27</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="2095500" cy="571500"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="25" name="Image 25" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId25"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>4</col>
+      <colOff>0</colOff>
+      <row>28</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="2095500" cy="571500"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="26" name="Image 26" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId26"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>4</col>
+      <colOff>0</colOff>
+      <row>29</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="2095500" cy="571500"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="27" name="Image 27" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId27"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>4</col>
+      <colOff>0</colOff>
+      <row>30</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="2095500" cy="571500"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="28" name="Image 28" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId28"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>4</col>
+      <colOff>0</colOff>
+      <row>31</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="2095500" cy="571500"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="29" name="Image 29" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId29"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>4</col>
+      <colOff>0</colOff>
+      <row>32</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="2095500" cy="571500"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="30" name="Image 30" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId30"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>4</col>
+      <colOff>0</colOff>
+      <row>33</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="2095500" cy="571500"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="31" name="Image 31" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId31"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+</wsDr>
+</file>
+
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
 <a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
   <a:themeElements>
@@ -6608,7 +8503,7 @@
     <col width="17.6" customWidth="1" min="13" max="13"/>
   </cols>
   <sheetData>
-    <row r="1" ht="32" customHeight="1">
+    <row r="1" ht="261" customHeight="1">
       <c r="A1" s="33" t="n"/>
       <c r="B1" s="34" t="inlineStr">
         <is>
@@ -8802,6 +10697,7 @@
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup orientation="landscape" fitToHeight="0" fitToWidth="1"/>
+  <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
 </worksheet>
 </file>
 
@@ -9801,7 +11697,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="5" ht="47" customHeight="1">
+    <row r="5" ht="48" customHeight="1">
       <c r="A5" s="37" t="n"/>
       <c r="B5" s="62" t="inlineStr">
         <is>
@@ -10013,7 +11909,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="7" ht="19.8" customHeight="1">
+    <row r="7" ht="48" customHeight="1">
       <c r="A7" s="37" t="n"/>
       <c r="B7" s="62" t="inlineStr">
         <is>
@@ -10225,7 +12121,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="9" ht="19.8" customHeight="1">
+    <row r="9" ht="48" customHeight="1">
       <c r="A9" s="37" t="n"/>
       <c r="B9" s="62" t="inlineStr">
         <is>
@@ -10437,7 +12333,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="11" ht="47" customHeight="1">
+    <row r="11" ht="48" customHeight="1">
       <c r="A11" s="37" t="n"/>
       <c r="B11" s="62" t="inlineStr">
         <is>
@@ -10543,7 +12439,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="12" ht="47" customHeight="1">
+    <row r="12" ht="48" customHeight="1">
       <c r="A12" s="37" t="n"/>
       <c r="B12" s="62" t="inlineStr">
         <is>
@@ -10759,7 +12655,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="14" ht="19.8" customHeight="1">
+    <row r="14" ht="48" customHeight="1">
       <c r="A14" s="37" t="n"/>
       <c r="B14" s="62" t="inlineStr">
         <is>
@@ -10861,7 +12757,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="15" ht="32" customHeight="1">
+    <row r="15" ht="48" customHeight="1">
       <c r="A15" s="37" t="n"/>
       <c r="B15" s="62" t="inlineStr">
         <is>
@@ -10967,7 +12863,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="16" ht="47" customHeight="1">
+    <row r="16" ht="48" customHeight="1">
       <c r="A16" s="37" t="n"/>
       <c r="B16" s="62" t="inlineStr">
         <is>
@@ -11081,7 +12977,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="17" ht="19.8" customHeight="1">
+    <row r="17" ht="48" customHeight="1">
       <c r="A17" s="37" t="n"/>
       <c r="B17" s="62" t="inlineStr">
         <is>
@@ -11183,7 +13079,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="18" ht="19.8" customHeight="1">
+    <row r="18" ht="48" customHeight="1">
       <c r="A18" s="37" t="n"/>
       <c r="B18" s="62" t="inlineStr">
         <is>
@@ -11285,7 +13181,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="19" ht="19.8" customHeight="1">
+    <row r="19" ht="48" customHeight="1">
       <c r="A19" s="37" t="n"/>
       <c r="B19" s="62" t="inlineStr">
         <is>
@@ -11493,7 +13389,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="21" ht="47" customHeight="1">
+    <row r="21" ht="48" customHeight="1">
       <c r="A21" s="37" t="n"/>
       <c r="B21" s="62" t="inlineStr">
         <is>
@@ -11599,7 +13495,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="22" ht="47" customHeight="1">
+    <row r="22" ht="48" customHeight="1">
       <c r="A22" s="37" t="n"/>
       <c r="B22" s="62" t="inlineStr">
         <is>
@@ -11813,7 +13709,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="24" ht="32" customHeight="1">
+    <row r="24" ht="48" customHeight="1">
       <c r="A24" s="37" t="n"/>
       <c r="B24" s="62" t="inlineStr">
         <is>
@@ -11919,7 +13815,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="25" ht="19.8" customHeight="1">
+    <row r="25" ht="48" customHeight="1">
       <c r="A25" s="5" t="n"/>
       <c r="B25" s="62" t="inlineStr">
         <is>
@@ -12029,7 +13925,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="26" ht="28.4" customHeight="1">
+    <row r="26" ht="48" customHeight="1">
       <c r="A26" s="8" t="inlineStr">
         <is>
           <t>TECHO</t>
@@ -12135,7 +14031,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="27" ht="19.8" customHeight="1">
+    <row r="27" ht="48" customHeight="1">
       <c r="A27" s="37" t="n"/>
       <c r="B27" s="62" t="inlineStr">
         <is>
@@ -12237,7 +14133,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="28" ht="19.8" customHeight="1">
+    <row r="28" ht="48" customHeight="1">
       <c r="A28" s="37" t="n"/>
       <c r="B28" s="62" t="inlineStr">
         <is>
@@ -12339,7 +14235,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="29" ht="19.8" customHeight="1">
+    <row r="29" ht="48" customHeight="1">
       <c r="A29" s="37" t="n"/>
       <c r="B29" s="62" t="inlineStr">
         <is>
@@ -12441,7 +14337,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="30" ht="47" customHeight="1">
+    <row r="30" ht="48" customHeight="1">
       <c r="A30" s="37" t="n"/>
       <c r="B30" s="62" t="inlineStr">
         <is>
@@ -12547,7 +14443,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="31" ht="47" customHeight="1">
+    <row r="31" ht="48" customHeight="1">
       <c r="A31" s="37" t="n"/>
       <c r="B31" s="62" t="inlineStr">
         <is>
@@ -12653,7 +14549,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="32" ht="19.8" customHeight="1">
+    <row r="32" ht="48" customHeight="1">
       <c r="A32" s="37" t="n"/>
       <c r="B32" s="62" t="inlineStr">
         <is>
@@ -12755,7 +14651,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="33" ht="19.8" customHeight="1">
+    <row r="33" ht="48" customHeight="1">
       <c r="A33" s="37" t="n"/>
       <c r="B33" s="62" t="inlineStr">
         <is>
@@ -12857,7 +14753,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="34" ht="19.8" customHeight="1">
+    <row r="34" ht="48" customHeight="1">
       <c r="A34" s="5" t="n"/>
       <c r="B34" s="63" t="inlineStr">
         <is>
@@ -12990,6 +14886,7 @@
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup orientation="landscape" fitToHeight="0" fitToWidth="1"/>
+  <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
 </worksheet>
 </file>
 
@@ -13179,7 +15076,7 @@
         </is>
       </c>
     </row>
-    <row r="4" ht="28.4" customHeight="1">
+    <row r="4" ht="48" customHeight="1">
       <c r="A4" s="8" t="inlineStr">
         <is>
           <t>S/PB</t>
@@ -13241,7 +15138,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="5" ht="19.8" customHeight="1">
+    <row r="5" ht="48" customHeight="1">
       <c r="A5" s="37" t="n"/>
       <c r="B5" s="62" t="inlineStr">
         <is>
@@ -13305,7 +15202,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="6" ht="19.8" customHeight="1">
+    <row r="6" ht="48" customHeight="1">
       <c r="A6" s="37" t="n"/>
       <c r="B6" s="62" t="inlineStr">
         <is>
@@ -13363,7 +15260,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="7" ht="19.8" customHeight="1">
+    <row r="7" ht="48" customHeight="1">
       <c r="A7" s="37" t="n"/>
       <c r="B7" s="62" t="inlineStr">
         <is>
@@ -13421,7 +15318,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="8" ht="19.8" customHeight="1">
+    <row r="8" ht="48" customHeight="1">
       <c r="A8" s="37" t="n"/>
       <c r="B8" s="62" t="inlineStr">
         <is>
@@ -13479,7 +15376,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="9" ht="19.8" customHeight="1">
+    <row r="9" ht="48" customHeight="1">
       <c r="A9" s="37" t="n"/>
       <c r="B9" s="62" t="inlineStr">
         <is>
@@ -13537,7 +15434,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="10" ht="47" customHeight="1">
+    <row r="10" ht="48" customHeight="1">
       <c r="A10" s="37" t="n"/>
       <c r="B10" s="62" t="inlineStr">
         <is>
@@ -13601,7 +15498,7 @@
         <v>0.639951021553631</v>
       </c>
     </row>
-    <row r="11" ht="32" customHeight="1">
+    <row r="11" ht="48" customHeight="1">
       <c r="A11" s="37" t="n"/>
       <c r="B11" s="62" t="inlineStr">
         <is>
@@ -13665,7 +15562,7 @@
         <v>0.360048978446369</v>
       </c>
     </row>
-    <row r="12" ht="19.8" customHeight="1">
+    <row r="12" ht="48" customHeight="1">
       <c r="A12" s="5" t="n"/>
       <c r="B12" s="62" t="inlineStr">
         <is>
@@ -13729,7 +15626,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="13" ht="28.4" customHeight="1">
+    <row r="13" ht="48" customHeight="1">
       <c r="A13" s="8" t="inlineStr">
         <is>
           <t>S/PA</t>
@@ -13791,7 +15688,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="14" ht="47" customHeight="1">
+    <row r="14" ht="48" customHeight="1">
       <c r="A14" s="37" t="n"/>
       <c r="B14" s="62" t="inlineStr">
         <is>
@@ -13855,7 +15752,7 @@
         <v>0.7008026762551089</v>
       </c>
     </row>
-    <row r="15" ht="32" customHeight="1">
+    <row r="15" ht="48" customHeight="1">
       <c r="A15" s="5" t="n"/>
       <c r="B15" s="63" t="inlineStr">
         <is>
@@ -13939,6 +15836,7 @@
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup orientation="landscape" fitToHeight="0" fitToWidth="1"/>
+  <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
 </worksheet>
 </file>
 
@@ -15151,7 +17049,7 @@
         </is>
       </c>
     </row>
-    <row r="4" ht="19.8" customHeight="1">
+    <row r="4" ht="48" customHeight="1">
       <c r="A4" s="56" t="inlineStr">
         <is>
           <t>VF01 (1)</t>
@@ -15233,7 +17131,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="5" ht="19.8" customHeight="1">
+    <row r="5" ht="48" customHeight="1">
       <c r="A5" s="56" t="inlineStr">
         <is>
           <t>VF01 (2)</t>
@@ -15315,7 +17213,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="6" ht="19.8" customHeight="1">
+    <row r="6" ht="48" customHeight="1">
       <c r="A6" s="56" t="inlineStr">
         <is>
           <t>VF01 (3)</t>
@@ -15397,7 +17295,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="7" ht="47" customHeight="1">
+    <row r="7" ht="48" customHeight="1">
       <c r="A7" s="56" t="inlineStr">
         <is>
           <t>VF02</t>
@@ -15665,7 +17563,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="10" ht="19.8" customHeight="1">
+    <row r="10" ht="48" customHeight="1">
       <c r="A10" s="56" t="inlineStr">
         <is>
           <t>VF04b</t>
@@ -15747,7 +17645,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="11" ht="19.8" customHeight="1">
+    <row r="11" ht="48" customHeight="1">
       <c r="A11" s="56" t="inlineStr">
         <is>
           <t>VF04c</t>
@@ -15829,7 +17727,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="12" ht="19.8" customHeight="1">
+    <row r="12" ht="48" customHeight="1">
       <c r="A12" s="56" t="inlineStr">
         <is>
           <t>VF05</t>
@@ -15919,7 +17817,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="13" ht="19.8" customHeight="1">
+    <row r="13" ht="48" customHeight="1">
       <c r="A13" s="56" t="inlineStr">
         <is>
           <t>VF06a</t>
@@ -16001,7 +17899,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="14" ht="19.8" customHeight="1">
+    <row r="14" ht="48" customHeight="1">
       <c r="A14" s="56" t="inlineStr">
         <is>
           <t>VF06b</t>
@@ -16083,7 +17981,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="15" ht="19.8" customHeight="1">
+    <row r="15" ht="48" customHeight="1">
       <c r="A15" s="56" t="inlineStr">
         <is>
           <t>VF06c</t>
@@ -16165,7 +18063,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="16" ht="19.8" customHeight="1">
+    <row r="16" ht="48" customHeight="1">
       <c r="A16" s="56" t="inlineStr">
         <is>
           <t>VF06d</t>
@@ -16247,7 +18145,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="17" ht="19.8" customHeight="1">
+    <row r="17" ht="48" customHeight="1">
       <c r="A17" s="56" t="inlineStr">
         <is>
           <t>VF07</t>
@@ -16337,7 +18235,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="18" ht="47" customHeight="1">
+    <row r="18" ht="48" customHeight="1">
       <c r="A18" s="56" t="inlineStr">
         <is>
           <t>VF08</t>
@@ -16431,7 +18329,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="19" ht="19.8" customHeight="1">
+    <row r="19" ht="48" customHeight="1">
       <c r="A19" s="56" t="inlineStr">
         <is>
           <t>VF09 (1)</t>
@@ -16513,7 +18411,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="20" ht="19.8" customHeight="1">
+    <row r="20" ht="48" customHeight="1">
       <c r="A20" s="56" t="inlineStr">
         <is>
           <t>VF09 (2)</t>
@@ -16595,7 +18493,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="21" ht="47" customHeight="1">
+    <row r="21" ht="48" customHeight="1">
       <c r="A21" s="56" t="inlineStr">
         <is>
           <t>VF10a</t>
@@ -16681,7 +18579,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="22" ht="47" customHeight="1">
+    <row r="22" ht="48" customHeight="1">
       <c r="A22" s="56" t="inlineStr">
         <is>
           <t>VF10b</t>
@@ -16767,7 +18665,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="23" ht="47" customHeight="1">
+    <row r="23" ht="48" customHeight="1">
       <c r="A23" s="56" t="inlineStr">
         <is>
           <t>VF10c</t>
@@ -16853,7 +18751,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="24" ht="47" customHeight="1">
+    <row r="24" ht="48" customHeight="1">
       <c r="A24" s="56" t="inlineStr">
         <is>
           <t>VF11</t>
@@ -16947,7 +18845,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="25" ht="19.8" customHeight="1">
+    <row r="25" ht="48" customHeight="1">
       <c r="A25" s="56" t="inlineStr">
         <is>
           <t>VF12</t>
@@ -17037,7 +18935,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="26" ht="19.8" customHeight="1">
+    <row r="26" ht="48" customHeight="1">
       <c r="A26" s="56" t="inlineStr">
         <is>
           <t>VF13</t>
@@ -17127,7 +19025,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="27" ht="47" customHeight="1">
+    <row r="27" ht="48" customHeight="1">
       <c r="A27" s="56" t="inlineStr">
         <is>
           <t>VF14</t>
@@ -17221,7 +19119,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="28" ht="19.8" customHeight="1">
+    <row r="28" ht="48" customHeight="1">
       <c r="A28" s="56" t="inlineStr">
         <is>
           <t>VF15</t>
@@ -17311,7 +19209,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="29" ht="47" customHeight="1">
+    <row r="29" ht="48" customHeight="1">
       <c r="A29" s="56" t="inlineStr">
         <is>
           <t>VF16a</t>
@@ -17397,7 +19295,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="30" ht="19.8" customHeight="1">
+    <row r="30" ht="48" customHeight="1">
       <c r="A30" s="56" t="inlineStr">
         <is>
           <t>VF16b</t>
@@ -17479,7 +19377,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="31" ht="19.8" customHeight="1">
+    <row r="31" ht="48" customHeight="1">
       <c r="A31" s="56" t="inlineStr">
         <is>
           <t>VF17</t>
@@ -17569,7 +19467,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="32" ht="47" customHeight="1">
+    <row r="32" ht="48" customHeight="1">
       <c r="A32" s="56" t="inlineStr">
         <is>
           <t>VF18a</t>
@@ -17655,7 +19553,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="33" ht="19.8" customHeight="1">
+    <row r="33" ht="48" customHeight="1">
       <c r="A33" s="56" t="inlineStr">
         <is>
           <t>VF18b</t>
@@ -17737,7 +19635,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="34" ht="47" customHeight="1">
+    <row r="34" ht="48" customHeight="1">
       <c r="A34" s="41" t="inlineStr">
         <is>
           <t>VF18c</t>
@@ -17843,6 +19741,7 @@
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup orientation="landscape" fitToHeight="0" fitToWidth="1"/>
+  <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
 </worksheet>
 </file>
 

</xml_diff>